<commit_message>
Fixed some error in the simulations.py
</commit_message>
<xml_diff>
--- a/ra/dataCounters/counters.xlsx
+++ b/ra/dataCounters/counters.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="A:\uni\masters nu\RA\pythonCode\ra\dataCounters\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F66BE00-EFAE-4E0B-899E-396410EEF85D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE2EFA1B-18CF-4EC1-81A8-E4C86F644E5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="24">
   <si>
     <t>num_links</t>
   </si>
@@ -88,12 +88,36 @@
   <si>
     <t>log_Ftst</t>
   </si>
+  <si>
+    <t>gibbs_AddCount</t>
+  </si>
+  <si>
+    <t>gibbs_MultCount</t>
+  </si>
+  <si>
+    <t>gibbs_TrigCount</t>
+  </si>
+  <si>
+    <t>lie_AddCount</t>
+  </si>
+  <si>
+    <t>lie_MultCount</t>
+  </si>
+  <si>
+    <t>lie_TrigCount</t>
+  </si>
+  <si>
+    <t>log_GA</t>
+  </si>
+  <si>
+    <t>log_lie</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -101,13 +125,68 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C5700"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.39997558519241921"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.39997558519241921"/>
+        <bgColor indexed="65"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -119,13 +198,28 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="3"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="4"/>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="5"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="6">
+    <cellStyle name="60% - Accent1" xfId="4" builtinId="32"/>
+    <cellStyle name="60% - Accent2" xfId="5" builtinId="36"/>
+    <cellStyle name="Bad" xfId="2" builtinId="27"/>
+    <cellStyle name="Good" xfId="1" builtinId="26"/>
+    <cellStyle name="Neutral" xfId="3" builtinId="28"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -784,6 +878,14 @@
           </a:p>
         </c:rich>
       </c:tx>
+      <c:layout>
+        <c:manualLayout>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.32340014204782686"/>
+          <c:y val="2.5574989763291499E-2"/>
+        </c:manualLayout>
+      </c:layout>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -905,7 +1007,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$O$2:$O$20</c:f>
+              <c:f>Sheet1!$AC$2:$AC$20</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="19"/>
@@ -1062,7 +1164,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$T$2:$T$20</c:f>
+              <c:f>Sheet1!$AH$2:$AH$20</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="19"/>
@@ -1219,7 +1321,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$Y$2:$Y$20</c:f>
+              <c:f>Sheet1!$AM$2:$AM$20</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="19"/>
@@ -1287,6 +1389,188 @@
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000002-0C58-405E-A377-7A3D7DD26BC5}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="3"/>
+          <c:order val="3"/>
+          <c:tx>
+            <c:v>GA Rot. Matrices</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent4"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet1!$AR$2:$AR$20</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="19"/>
+                <c:pt idx="0">
+                  <c:v>0.77815125038364363</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.95424250943932487</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1.0791812460476249</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1.1760912590556813</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1.255272505103306</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1.3222192947339193</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1.3802112417116059</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>1.4313637641589874</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>1.4771212547196624</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>1.5185139398778875</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>1.5563025007672873</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>1.5910646070264991</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>1.6232492903979006</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>1.6532125137753437</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>1.6812412373755872</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>1.7075701760979363</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>1.7323937598229686</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>1.7558748556724915</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>1.7781512503836436</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-E6DC-410D-BBCC-A5C1B3C3438C}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="4"/>
+          <c:order val="4"/>
+          <c:tx>
+            <c:v>Lie Group Rot. Matrices</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent6"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet1!$AW$2:$AW$20</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="19"/>
+                <c:pt idx="0">
+                  <c:v>0.84509804001425681</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1.0413926851582251</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1.1760912590556813</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1.2787536009528289</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1.3617278360175928</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1.4313637641589874</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1.4913616938342726</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>1.5440680443502757</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>1.5910646070264991</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>1.6334684555795864</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>1.6720978579357175</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>1.7075701760979363</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>1.7403626894942439</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>1.7708520116421442</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>1.7993405494535817</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>1.8260748027008264</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>1.8512583487190752</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>1.8750612633917001</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>1.8976270912904414</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-E6DC-410D-BBCC-A5C1B3C3438C}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1550,8 +1834,8 @@
           <c:yMode val="edge"/>
           <c:x val="0.1210531614790612"/>
           <c:y val="0.13356479174280428"/>
-          <c:w val="0.15576215216764974"/>
-          <c:h val="0.19585191091619877"/>
+          <c:w val="0.21359291377421535"/>
+          <c:h val="0.23976720717979241"/>
         </c:manualLayout>
       </c:layout>
       <c:overlay val="1"/>
@@ -5688,7 +5972,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$M$2:$M$20</c:f>
+              <c:f>Sheet1!$AA$2:$AA$20</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="19"/>
@@ -5845,7 +6129,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$R$2:$R$20</c:f>
+              <c:f>Sheet1!$AF$2:$AF$20</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="19"/>
@@ -6002,7 +6286,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$W$2:$W$20</c:f>
+              <c:f>Sheet1!$AK$2:$AK$20</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="19"/>
@@ -6070,6 +6354,188 @@
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000002-7782-48BD-A375-0041F112F0CE}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="3"/>
+          <c:order val="3"/>
+          <c:tx>
+            <c:v>GA Add</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent4"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet1!$AP$2:$AP$20</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="19"/>
+                <c:pt idx="0">
+                  <c:v>1.4771212547196624</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1.6532125137753437</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1.7781512503836436</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1.8750612633917001</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1.954242509439325</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>2.0211892990699383</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>2.0791812460476247</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>2.1303337684950061</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>2.1760912590556813</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>2.2174839442139063</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>2.255272505103306</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>2.2900346113625178</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>2.3222192947339191</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>2.3521825181113627</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>2.3802112417116059</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>2.406540180433955</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>2.4313637641589874</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>2.4548448600085102</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>2.4771212547196626</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-978B-47B5-A9C7-E47B4C75958F}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="4"/>
+          <c:order val="4"/>
+          <c:tx>
+            <c:v>Lie Group Add</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent6"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet1!$AU$2:$AU$21</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>1.1139433523068367</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1.3010299956639813</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1.4313637641589874</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1.5314789170422551</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1.6127838567197355</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1.6812412373755872</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1.7403626894942439</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>1.7923916894982539</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>1.8388490907372552</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>1.8808135922807914</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>1.919078092376074</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>1.954242509439325</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>1.9867717342662448</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>2.0170333392987803</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>2.0453229787866576</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>2.0718820073061255</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>2.0969100130080562</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>2.12057393120585</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>2.143014800254095</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-978B-47B5-A9C7-E47B4C75958F}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -6322,8 +6788,8 @@
           <c:yMode val="edge"/>
           <c:x val="0.18056261061456588"/>
           <c:y val="0.170133005526208"/>
-          <c:w val="0.15576215216764974"/>
-          <c:h val="0.14240606000199343"/>
+          <c:w val="0.15688977522976036"/>
+          <c:h val="0.23987374712489298"/>
         </c:manualLayout>
       </c:layout>
       <c:overlay val="1"/>
@@ -6563,7 +7029,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$R$2:$R$20</c:f>
+              <c:f>Sheet1!$AF$2:$AF$20</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="19"/>
@@ -6717,7 +7183,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$M$2:$M$20</c:f>
+              <c:f>Sheet1!$AA$2:$AA$20</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="19"/>
@@ -6871,7 +7337,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$W$2:$W$20</c:f>
+              <c:f>Sheet1!$AK$2:$AK$20</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="19"/>
@@ -7438,7 +7904,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$N$2:$N$20</c:f>
+              <c:f>Sheet1!$AB$2:$AB$20</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="19"/>
@@ -7595,7 +8061,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$S$2:$S$20</c:f>
+              <c:f>Sheet1!$AG$2:$AG$20</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="19"/>
@@ -7752,7 +8218,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$X$2:$X$20</c:f>
+              <c:f>Sheet1!$AL$2:$AL$20</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="19"/>
@@ -7820,6 +8286,188 @@
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000002-F1F7-458C-87BB-5B7EA60AD675}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="3"/>
+          <c:order val="3"/>
+          <c:tx>
+            <c:v>GA Multiplication</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent4"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet1!$AQ$2:$AQ$20</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="19"/>
+                <c:pt idx="0">
+                  <c:v>1.6020599913279623</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1.7781512503836436</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1.9030899869919435</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>2.0791812460476247</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>2.1461280356782382</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>2.2041199826559246</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>2.255272505103306</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>2.3010299956639813</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>2.3424226808222062</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>2.3802112417116059</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>2.4149733479708178</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>2.4471580313422194</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>2.4771212547196626</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>2.5051499783199058</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>2.5314789170422549</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>2.5563025007672873</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>2.5797835966168101</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>2.6020599913279625</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-F210-46B0-97CD-141395340F13}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="4"/>
+          <c:order val="4"/>
+          <c:tx>
+            <c:v>Lie Group Multiplication</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent6"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet1!$AV$2:$AV$20</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="19"/>
+                <c:pt idx="0">
+                  <c:v>1.3979400086720377</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1.5797835966168101</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1.7075701760979363</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1.8061799739838871</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1.8864907251724818</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1.954242509439325</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>2.012837224705172</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>2.0644579892269186</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>2.1105897102992488</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>2.1522883443830563</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>2.1903316981702914</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>2.2253092817258628</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>2.2576785748691846</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>2.287801729930226</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>2.3159703454569178</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>2.3424226808222062</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>2.3673559210260189</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>2.3909351071033793</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>2.4132997640812519</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-F210-46B0-97CD-141395340F13}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -8072,8 +8720,8 @@
           <c:yMode val="edge"/>
           <c:x val="0.1210531614790612"/>
           <c:y val="0.13356479174280428"/>
-          <c:w val="0.15576215216764974"/>
-          <c:h val="0.19585191091619877"/>
+          <c:w val="0.22358559351956353"/>
+          <c:h val="0.23976726082848218"/>
         </c:manualLayout>
       </c:layout>
       <c:overlay val="1"/>
@@ -14040,16 +14688,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>20</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>85</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>128984</xdr:colOff>
+      <xdr:row>84</xdr:row>
+      <xdr:rowOff>49609</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>32</xdr:col>
-      <xdr:colOff>581025</xdr:colOff>
-      <xdr:row>108</xdr:row>
-      <xdr:rowOff>133350</xdr:rowOff>
+      <xdr:col>31</xdr:col>
+      <xdr:colOff>104774</xdr:colOff>
+      <xdr:row>107</xdr:row>
+      <xdr:rowOff>182960</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -14101,8 +14749,8 @@
       <sheetName val="90s 9000"/>
     </sheetNames>
     <sheetDataSet>
-      <sheetData sheetId="0" refreshError="1"/>
-      <sheetData sheetId="1" refreshError="1"/>
+      <sheetData sheetId="0"/>
+      <sheetData sheetId="1"/>
       <sheetData sheetId="2">
         <row r="2">
           <cell r="A2">
@@ -14200,15 +14848,15 @@
           </cell>
         </row>
       </sheetData>
-      <sheetData sheetId="3" refreshError="1"/>
-      <sheetData sheetId="4" refreshError="1"/>
-      <sheetData sheetId="5" refreshError="1"/>
-      <sheetData sheetId="6" refreshError="1"/>
-      <sheetData sheetId="7" refreshError="1"/>
-      <sheetData sheetId="8" refreshError="1"/>
-      <sheetData sheetId="9" refreshError="1"/>
-      <sheetData sheetId="10" refreshError="1"/>
-      <sheetData sheetId="11" refreshError="1"/>
+      <sheetData sheetId="3"/>
+      <sheetData sheetId="4"/>
+      <sheetData sheetId="5"/>
+      <sheetData sheetId="6"/>
+      <sheetData sheetId="7"/>
+      <sheetData sheetId="8"/>
+      <sheetData sheetId="9"/>
+      <sheetData sheetId="10"/>
+      <sheetData sheetId="11"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -14477,7 +15125,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Y20"/>
+  <dimension ref="A1:AW21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.7109375" customWidth="1"/>
@@ -14490,1367 +15138,2218 @@
     <col min="8" max="8" width="21.28515625" customWidth="1"/>
     <col min="9" max="9" width="21.7109375" customWidth="1"/>
     <col min="10" max="10" width="30" customWidth="1"/>
+    <col min="11" max="11" width="16" customWidth="1"/>
+    <col min="12" max="12" width="23.85546875" customWidth="1"/>
+    <col min="13" max="13" width="17.5703125" customWidth="1"/>
+    <col min="14" max="14" width="14" customWidth="1"/>
+    <col min="15" max="15" width="17.5703125" customWidth="1"/>
+    <col min="16" max="16" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="L1" t="s">
+      <c r="K1" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="L1" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="M1" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="N1" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="O1" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="P1" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="Z1" t="s">
         <v>13</v>
       </c>
-      <c r="M1" t="s">
+      <c r="AA1" t="s">
         <v>10</v>
       </c>
-      <c r="N1" t="s">
+      <c r="AB1" t="s">
         <v>11</v>
       </c>
-      <c r="O1" t="s">
+      <c r="AC1" t="s">
         <v>12</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="AE1" t="s">
         <v>14</v>
       </c>
-      <c r="R1" t="s">
+      <c r="AF1" t="s">
         <v>10</v>
       </c>
-      <c r="S1" t="s">
+      <c r="AG1" t="s">
         <v>11</v>
       </c>
-      <c r="T1" t="s">
+      <c r="AH1" t="s">
         <v>12</v>
       </c>
-      <c r="V1" t="s">
+      <c r="AJ1" t="s">
         <v>15</v>
       </c>
-      <c r="W1" t="s">
+      <c r="AK1" t="s">
         <v>10</v>
       </c>
-      <c r="X1" t="s">
+      <c r="AL1" t="s">
         <v>11</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="AM1" t="s">
         <v>12</v>
       </c>
+      <c r="AO1" t="s">
+        <v>22</v>
+      </c>
+      <c r="AP1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AQ1" t="s">
+        <v>11</v>
+      </c>
+      <c r="AR1" t="s">
+        <v>12</v>
+      </c>
+      <c r="AT1" t="s">
+        <v>23</v>
+      </c>
+      <c r="AU1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AV1" t="s">
+        <v>11</v>
+      </c>
+      <c r="AW1" t="s">
+        <v>12</v>
+      </c>
     </row>
-    <row r="2" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>2</v>
       </c>
-      <c r="B2">
+      <c r="B2" s="1">
         <v>20</v>
       </c>
-      <c r="C2">
+      <c r="C2" s="1">
         <v>113</v>
       </c>
-      <c r="D2">
+      <c r="D2" s="1">
         <v>141</v>
       </c>
-      <c r="E2">
+      <c r="E2" s="2">
         <v>22</v>
       </c>
-      <c r="F2">
+      <c r="F2" s="2">
         <v>39</v>
       </c>
-      <c r="G2">
+      <c r="G2" s="2">
         <v>6</v>
       </c>
-      <c r="H2">
+      <c r="H2" s="3">
         <v>11</v>
       </c>
-      <c r="I2">
+      <c r="I2" s="3">
         <v>24</v>
       </c>
-      <c r="J2">
+      <c r="J2" s="3">
         <v>2</v>
       </c>
-      <c r="M2">
+      <c r="K2" s="4">
+        <v>30</v>
+      </c>
+      <c r="L2" s="4">
+        <v>40</v>
+      </c>
+      <c r="M2" s="4">
+        <v>6</v>
+      </c>
+      <c r="N2" s="5">
+        <v>13</v>
+      </c>
+      <c r="O2" s="5">
+        <v>25</v>
+      </c>
+      <c r="P2" s="5">
+        <v>7</v>
+      </c>
+      <c r="AA2">
         <f>LOG(B2)</f>
         <v>1.3010299956639813</v>
       </c>
-      <c r="N2">
-        <f t="shared" ref="N2:O17" si="0">LOG(C2)</f>
+      <c r="AB2">
+        <f>LOG(C2)</f>
         <v>2.0530784434834195</v>
       </c>
-      <c r="O2">
-        <f t="shared" si="0"/>
+      <c r="AC2">
+        <f>LOG(D2)</f>
         <v>2.1492191126553797</v>
       </c>
-      <c r="R2">
+      <c r="AF2">
         <f>LOG(E2)</f>
         <v>1.3424226808222062</v>
       </c>
-      <c r="S2">
-        <f t="shared" ref="S2:T17" si="1">LOG(F2)</f>
+      <c r="AG2">
+        <f>LOG(F2)</f>
         <v>1.5910646070264991</v>
       </c>
-      <c r="T2">
-        <f t="shared" si="1"/>
+      <c r="AH2">
+        <f>LOG(G2)</f>
         <v>0.77815125038364363</v>
       </c>
-      <c r="W2">
+      <c r="AK2">
         <f>LOG(H2)</f>
         <v>1.0413926851582251</v>
       </c>
-      <c r="X2">
-        <f t="shared" ref="X2:Y17" si="2">LOG(I2)</f>
+      <c r="AL2">
+        <f>LOG(I2)</f>
         <v>1.3802112417116059</v>
       </c>
-      <c r="Y2">
-        <f t="shared" si="2"/>
+      <c r="AM2">
+        <f>LOG(J2)</f>
         <v>0.3010299956639812</v>
       </c>
+      <c r="AP2">
+        <f>LOG(K2)</f>
+        <v>1.4771212547196624</v>
+      </c>
+      <c r="AQ2">
+        <f t="shared" ref="AQ2:AR17" si="0">LOG(L2)</f>
+        <v>1.6020599913279623</v>
+      </c>
+      <c r="AR2">
+        <f t="shared" si="0"/>
+        <v>0.77815125038364363</v>
+      </c>
+      <c r="AU2">
+        <f>LOG(N2)</f>
+        <v>1.1139433523068367</v>
+      </c>
+      <c r="AV2">
+        <f t="shared" ref="AV2:AW17" si="1">LOG(O2)</f>
+        <v>1.3979400086720377</v>
+      </c>
+      <c r="AW2">
+        <f t="shared" si="1"/>
+        <v>0.84509804001425681</v>
+      </c>
     </row>
-    <row r="3" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>3</v>
       </c>
-      <c r="B3">
+      <c r="B3" s="1">
         <v>59</v>
       </c>
-      <c r="C3">
+      <c r="C3" s="1">
         <v>494</v>
       </c>
-      <c r="D3">
+      <c r="D3" s="1">
         <v>642</v>
       </c>
-      <c r="E3">
+      <c r="E3" s="2">
         <v>36</v>
       </c>
-      <c r="F3">
+      <c r="F3" s="2">
         <v>63</v>
       </c>
-      <c r="G3">
+      <c r="G3" s="2">
         <v>11</v>
       </c>
-      <c r="H3">
+      <c r="H3" s="3">
         <v>18</v>
       </c>
-      <c r="I3">
+      <c r="I3" s="3">
         <v>37</v>
       </c>
-      <c r="J3">
+      <c r="J3" s="3">
         <v>3</v>
       </c>
-      <c r="M3">
-        <f t="shared" ref="M3:M20" si="3">LOG(B3)</f>
+      <c r="K3" s="4">
+        <v>45</v>
+      </c>
+      <c r="L3" s="4">
+        <v>60</v>
+      </c>
+      <c r="M3" s="4">
+        <v>9</v>
+      </c>
+      <c r="N3" s="5">
+        <v>20</v>
+      </c>
+      <c r="O3" s="5">
+        <v>38</v>
+      </c>
+      <c r="P3" s="5">
+        <v>11</v>
+      </c>
+      <c r="AA3">
+        <f>LOG(B3)</f>
         <v>1.7708520116421442</v>
       </c>
-      <c r="N3">
+      <c r="AB3">
+        <f>LOG(C3)</f>
+        <v>2.6937269489236471</v>
+      </c>
+      <c r="AC3">
+        <f>LOG(D3)</f>
+        <v>2.8075350280688531</v>
+      </c>
+      <c r="AF3">
+        <f>LOG(E3)</f>
+        <v>1.5563025007672873</v>
+      </c>
+      <c r="AG3">
+        <f>LOG(F3)</f>
+        <v>1.7993405494535817</v>
+      </c>
+      <c r="AH3">
+        <f>LOG(G3)</f>
+        <v>1.0413926851582251</v>
+      </c>
+      <c r="AK3">
+        <f>LOG(H3)</f>
+        <v>1.255272505103306</v>
+      </c>
+      <c r="AL3">
+        <f>LOG(I3)</f>
+        <v>1.568201724066995</v>
+      </c>
+      <c r="AM3">
+        <f>LOG(J3)</f>
+        <v>0.47712125471966244</v>
+      </c>
+      <c r="AP3">
+        <f t="shared" ref="AP3:AP20" si="2">LOG(K3)</f>
+        <v>1.6532125137753437</v>
+      </c>
+      <c r="AQ3">
         <f t="shared" si="0"/>
-        <v>2.6937269489236471</v>
-      </c>
-      <c r="O3">
+        <v>1.7781512503836436</v>
+      </c>
+      <c r="AR3">
         <f t="shared" si="0"/>
-        <v>2.8075350280688531</v>
-      </c>
-      <c r="R3">
-        <f t="shared" ref="R3:R20" si="4">LOG(E3)</f>
+        <v>0.95424250943932487</v>
+      </c>
+      <c r="AU3">
+        <f t="shared" ref="AU3:AU20" si="3">LOG(N3)</f>
+        <v>1.3010299956639813</v>
+      </c>
+      <c r="AV3">
+        <f t="shared" si="1"/>
+        <v>1.5797835966168101</v>
+      </c>
+      <c r="AW3">
+        <f t="shared" si="1"/>
+        <v>1.0413926851582251</v>
+      </c>
+    </row>
+    <row r="4" spans="1:49" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>4</v>
+      </c>
+      <c r="B4" s="1">
+        <v>143</v>
+      </c>
+      <c r="C4" s="1">
+        <v>1526</v>
+      </c>
+      <c r="D4" s="1">
+        <v>2038</v>
+      </c>
+      <c r="E4" s="2">
+        <v>50</v>
+      </c>
+      <c r="F4" s="2">
+        <v>88</v>
+      </c>
+      <c r="G4" s="2">
+        <v>17</v>
+      </c>
+      <c r="H4" s="3">
+        <v>25</v>
+      </c>
+      <c r="I4" s="3">
+        <v>50</v>
+      </c>
+      <c r="J4" s="3">
+        <v>4</v>
+      </c>
+      <c r="K4" s="4">
+        <v>60</v>
+      </c>
+      <c r="L4" s="4">
+        <v>80</v>
+      </c>
+      <c r="M4" s="4">
+        <v>12</v>
+      </c>
+      <c r="N4" s="5">
+        <v>27</v>
+      </c>
+      <c r="O4" s="5">
+        <v>51</v>
+      </c>
+      <c r="P4" s="5">
+        <v>15</v>
+      </c>
+      <c r="AA4">
+        <f>LOG(B4)</f>
+        <v>2.1553360374650619</v>
+      </c>
+      <c r="AB4">
+        <f>LOG(C4)</f>
+        <v>3.1835545336188615</v>
+      </c>
+      <c r="AC4">
+        <f>LOG(D4)</f>
+        <v>3.3092041796704077</v>
+      </c>
+      <c r="AF4">
+        <f>LOG(E4)</f>
+        <v>1.6989700043360187</v>
+      </c>
+      <c r="AG4">
+        <f>LOG(F4)</f>
+        <v>1.9444826721501687</v>
+      </c>
+      <c r="AH4">
+        <f>LOG(G4)</f>
+        <v>1.2304489213782739</v>
+      </c>
+      <c r="AK4">
+        <f>LOG(H4)</f>
+        <v>1.3979400086720377</v>
+      </c>
+      <c r="AL4">
+        <f>LOG(I4)</f>
+        <v>1.6989700043360187</v>
+      </c>
+      <c r="AM4">
+        <f>LOG(J4)</f>
+        <v>0.6020599913279624</v>
+      </c>
+      <c r="AP4">
+        <f t="shared" si="2"/>
+        <v>1.7781512503836436</v>
+      </c>
+      <c r="AQ4">
+        <f t="shared" si="0"/>
+        <v>1.9030899869919435</v>
+      </c>
+      <c r="AR4">
+        <f t="shared" si="0"/>
+        <v>1.0791812460476249</v>
+      </c>
+      <c r="AU4">
+        <f t="shared" si="3"/>
+        <v>1.4313637641589874</v>
+      </c>
+      <c r="AV4">
+        <f t="shared" si="1"/>
+        <v>1.7075701760979363</v>
+      </c>
+      <c r="AW4">
+        <f t="shared" si="1"/>
+        <v>1.1760912590556813</v>
+      </c>
+    </row>
+    <row r="5" spans="1:49" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>5</v>
+      </c>
+      <c r="B5" s="1">
+        <v>298</v>
+      </c>
+      <c r="C5" s="1">
+        <v>3791</v>
+      </c>
+      <c r="D5" s="1">
+        <v>5193</v>
+      </c>
+      <c r="E5" s="2">
+        <v>64</v>
+      </c>
+      <c r="F5" s="2">
+        <v>114</v>
+      </c>
+      <c r="G5" s="2">
+        <v>24</v>
+      </c>
+      <c r="H5" s="3">
+        <v>32</v>
+      </c>
+      <c r="I5" s="3">
+        <v>63</v>
+      </c>
+      <c r="J5" s="3">
+        <v>5</v>
+      </c>
+      <c r="K5" s="4">
+        <v>75</v>
+      </c>
+      <c r="L5" s="4">
+        <v>100</v>
+      </c>
+      <c r="M5" s="4">
+        <v>15</v>
+      </c>
+      <c r="N5" s="5">
+        <v>34</v>
+      </c>
+      <c r="O5" s="5">
+        <v>64</v>
+      </c>
+      <c r="P5" s="5">
+        <v>19</v>
+      </c>
+      <c r="AA5">
+        <f>LOG(B5)</f>
+        <v>2.4742162640762553</v>
+      </c>
+      <c r="AB5">
+        <f>LOG(C5)</f>
+        <v>3.5787537844264348</v>
+      </c>
+      <c r="AC5">
+        <f>LOG(D5)</f>
+        <v>3.7154183225950561</v>
+      </c>
+      <c r="AF5">
+        <f>LOG(E5)</f>
+        <v>1.8061799739838871</v>
+      </c>
+      <c r="AG5">
+        <f>LOG(F5)</f>
+        <v>2.0569048513364727</v>
+      </c>
+      <c r="AH5">
+        <f>LOG(G5)</f>
+        <v>1.3802112417116059</v>
+      </c>
+      <c r="AK5">
+        <f>LOG(H5)</f>
+        <v>1.505149978319906</v>
+      </c>
+      <c r="AL5">
+        <f>LOG(I5)</f>
+        <v>1.7993405494535817</v>
+      </c>
+      <c r="AM5">
+        <f>LOG(J5)</f>
+        <v>0.69897000433601886</v>
+      </c>
+      <c r="AP5">
+        <f t="shared" si="2"/>
+        <v>1.8750612633917001</v>
+      </c>
+      <c r="AQ5">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="AR5">
+        <f t="shared" si="0"/>
+        <v>1.1760912590556813</v>
+      </c>
+      <c r="AU5">
+        <f t="shared" si="3"/>
+        <v>1.5314789170422551</v>
+      </c>
+      <c r="AV5">
+        <f t="shared" si="1"/>
+        <v>1.8061799739838871</v>
+      </c>
+      <c r="AW5">
+        <f t="shared" si="1"/>
+        <v>1.2787536009528289</v>
+      </c>
+    </row>
+    <row r="6" spans="1:49" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>6</v>
+      </c>
+      <c r="B6" s="1">
+        <v>556</v>
+      </c>
+      <c r="C6" s="1">
+        <v>8135</v>
+      </c>
+      <c r="D6" s="1">
+        <v>11403</v>
+      </c>
+      <c r="E6" s="2">
+        <v>78</v>
+      </c>
+      <c r="F6" s="2">
+        <v>141</v>
+      </c>
+      <c r="G6" s="2">
+        <v>32</v>
+      </c>
+      <c r="H6" s="3">
+        <v>39</v>
+      </c>
+      <c r="I6" s="3">
+        <v>76</v>
+      </c>
+      <c r="J6" s="3">
+        <v>6</v>
+      </c>
+      <c r="K6" s="4">
+        <v>90</v>
+      </c>
+      <c r="L6" s="4">
+        <v>120</v>
+      </c>
+      <c r="M6" s="4">
+        <v>18</v>
+      </c>
+      <c r="N6" s="5">
+        <v>41</v>
+      </c>
+      <c r="O6" s="5">
+        <v>77</v>
+      </c>
+      <c r="P6" s="5">
+        <v>23</v>
+      </c>
+      <c r="AA6">
+        <f>LOG(B6)</f>
+        <v>2.7450747915820575</v>
+      </c>
+      <c r="AB6">
+        <f>LOG(C6)</f>
+        <v>3.9103575572728775</v>
+      </c>
+      <c r="AC6">
+        <f>LOG(D6)</f>
+        <v>4.0570191243227658</v>
+      </c>
+      <c r="AF6">
+        <f>LOG(E6)</f>
+        <v>1.8920946026904804</v>
+      </c>
+      <c r="AG6">
+        <f>LOG(F6)</f>
+        <v>2.1492191126553797</v>
+      </c>
+      <c r="AH6">
+        <f>LOG(G6)</f>
+        <v>1.505149978319906</v>
+      </c>
+      <c r="AK6">
+        <f>LOG(H6)</f>
+        <v>1.5910646070264991</v>
+      </c>
+      <c r="AL6">
+        <f>LOG(I6)</f>
+        <v>1.8808135922807914</v>
+      </c>
+      <c r="AM6">
+        <f>LOG(J6)</f>
+        <v>0.77815125038364363</v>
+      </c>
+      <c r="AP6">
+        <f t="shared" si="2"/>
+        <v>1.954242509439325</v>
+      </c>
+      <c r="AQ6">
+        <f t="shared" si="0"/>
+        <v>2.0791812460476247</v>
+      </c>
+      <c r="AR6">
+        <f t="shared" si="0"/>
+        <v>1.255272505103306</v>
+      </c>
+      <c r="AU6">
+        <f t="shared" si="3"/>
+        <v>1.6127838567197355</v>
+      </c>
+      <c r="AV6">
+        <f t="shared" si="1"/>
+        <v>1.8864907251724818</v>
+      </c>
+      <c r="AW6">
+        <f t="shared" si="1"/>
+        <v>1.3617278360175928</v>
+      </c>
+    </row>
+    <row r="7" spans="1:49" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>7</v>
+      </c>
+      <c r="B7" s="1">
+        <v>955</v>
+      </c>
+      <c r="C7" s="1">
+        <v>15716</v>
+      </c>
+      <c r="D7" s="1">
+        <v>22484</v>
+      </c>
+      <c r="E7" s="2">
+        <v>92</v>
+      </c>
+      <c r="F7" s="2">
+        <v>169</v>
+      </c>
+      <c r="G7" s="2">
+        <v>41</v>
+      </c>
+      <c r="H7" s="3">
+        <v>46</v>
+      </c>
+      <c r="I7" s="3">
+        <v>89</v>
+      </c>
+      <c r="J7" s="3">
+        <v>7</v>
+      </c>
+      <c r="K7" s="4">
+        <v>105</v>
+      </c>
+      <c r="L7" s="4">
+        <v>140</v>
+      </c>
+      <c r="M7" s="4">
+        <v>21</v>
+      </c>
+      <c r="N7" s="5">
+        <v>48</v>
+      </c>
+      <c r="O7" s="5">
+        <v>90</v>
+      </c>
+      <c r="P7" s="5">
+        <v>27</v>
+      </c>
+      <c r="AA7">
+        <f>LOG(B7)</f>
+        <v>2.9800033715837464</v>
+      </c>
+      <c r="AB7">
+        <f>LOG(C7)</f>
+        <v>4.1963420201397685</v>
+      </c>
+      <c r="AC7">
+        <f>LOG(D7)</f>
+        <v>4.3518735766208998</v>
+      </c>
+      <c r="AF7">
+        <f>LOG(E7)</f>
+        <v>1.9637878273455553</v>
+      </c>
+      <c r="AG7">
+        <f>LOG(F7)</f>
+        <v>2.2278867046136734</v>
+      </c>
+      <c r="AH7">
+        <f>LOG(G7)</f>
+        <v>1.6127838567197355</v>
+      </c>
+      <c r="AK7">
+        <f>LOG(H7)</f>
+        <v>1.6627578316815741</v>
+      </c>
+      <c r="AL7">
+        <f>LOG(I7)</f>
+        <v>1.9493900066449128</v>
+      </c>
+      <c r="AM7">
+        <f>LOG(J7)</f>
+        <v>0.84509804001425681</v>
+      </c>
+      <c r="AP7">
+        <f t="shared" si="2"/>
+        <v>2.0211892990699383</v>
+      </c>
+      <c r="AQ7">
+        <f t="shared" si="0"/>
+        <v>2.1461280356782382</v>
+      </c>
+      <c r="AR7">
+        <f t="shared" si="0"/>
+        <v>1.3222192947339193</v>
+      </c>
+      <c r="AU7">
+        <f t="shared" si="3"/>
+        <v>1.6812412373755872</v>
+      </c>
+      <c r="AV7">
+        <f t="shared" si="1"/>
+        <v>1.954242509439325</v>
+      </c>
+      <c r="AW7">
+        <f t="shared" si="1"/>
+        <v>1.4313637641589874</v>
+      </c>
+    </row>
+    <row r="8" spans="1:49" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>8</v>
+      </c>
+      <c r="B8" s="1">
+        <v>1539</v>
+      </c>
+      <c r="C8" s="1">
+        <v>28052</v>
+      </c>
+      <c r="D8" s="1">
+        <v>40860</v>
+      </c>
+      <c r="E8" s="2">
+        <v>106</v>
+      </c>
+      <c r="F8" s="2">
+        <v>198</v>
+      </c>
+      <c r="G8" s="2">
+        <v>51</v>
+      </c>
+      <c r="H8" s="3">
+        <v>53</v>
+      </c>
+      <c r="I8" s="3">
+        <v>102</v>
+      </c>
+      <c r="J8" s="3">
+        <v>8</v>
+      </c>
+      <c r="K8" s="4">
+        <v>120</v>
+      </c>
+      <c r="L8" s="4">
+        <v>160</v>
+      </c>
+      <c r="M8" s="4">
+        <v>24</v>
+      </c>
+      <c r="N8" s="5">
+        <v>55</v>
+      </c>
+      <c r="O8" s="5">
+        <v>103</v>
+      </c>
+      <c r="P8" s="5">
+        <v>31</v>
+      </c>
+      <c r="AA8">
+        <f>LOG(B8)</f>
+        <v>3.1872386198314788</v>
+      </c>
+      <c r="AB8">
+        <f>LOG(C8)</f>
+        <v>4.4479638302267448</v>
+      </c>
+      <c r="AC8">
+        <f>LOG(D8)</f>
+        <v>4.611298362296429</v>
+      </c>
+      <c r="AF8">
+        <f>LOG(E8)</f>
+        <v>2.0253058652647704</v>
+      </c>
+      <c r="AG8">
+        <f>LOG(F8)</f>
+        <v>2.2966651902615309</v>
+      </c>
+      <c r="AH8">
+        <f>LOG(G8)</f>
+        <v>1.7075701760979363</v>
+      </c>
+      <c r="AK8">
+        <f>LOG(H8)</f>
+        <v>1.7242758696007889</v>
+      </c>
+      <c r="AL8">
+        <f>LOG(I8)</f>
+        <v>2.0086001717619175</v>
+      </c>
+      <c r="AM8">
+        <f>LOG(J8)</f>
+        <v>0.90308998699194354</v>
+      </c>
+      <c r="AP8">
+        <f t="shared" si="2"/>
+        <v>2.0791812460476247</v>
+      </c>
+      <c r="AQ8">
+        <f t="shared" si="0"/>
+        <v>2.2041199826559246</v>
+      </c>
+      <c r="AR8">
+        <f t="shared" si="0"/>
+        <v>1.3802112417116059</v>
+      </c>
+      <c r="AU8">
+        <f t="shared" si="3"/>
+        <v>1.7403626894942439</v>
+      </c>
+      <c r="AV8">
+        <f t="shared" si="1"/>
+        <v>2.012837224705172</v>
+      </c>
+      <c r="AW8">
+        <f t="shared" si="1"/>
+        <v>1.4913616938342726</v>
+      </c>
+    </row>
+    <row r="9" spans="1:49" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>9</v>
+      </c>
+      <c r="B9" s="1">
+        <v>2358</v>
+      </c>
+      <c r="C9" s="1">
+        <v>47069</v>
+      </c>
+      <c r="D9" s="1">
+        <v>69651</v>
+      </c>
+      <c r="E9" s="2">
+        <v>120</v>
+      </c>
+      <c r="F9" s="2">
+        <v>228</v>
+      </c>
+      <c r="G9" s="2">
+        <v>62</v>
+      </c>
+      <c r="H9" s="3">
+        <v>60</v>
+      </c>
+      <c r="I9" s="3">
+        <v>115</v>
+      </c>
+      <c r="J9" s="3">
+        <v>9</v>
+      </c>
+      <c r="K9" s="4">
+        <v>135</v>
+      </c>
+      <c r="L9" s="4">
+        <v>180</v>
+      </c>
+      <c r="M9" s="4">
+        <v>27</v>
+      </c>
+      <c r="N9" s="5">
+        <v>62</v>
+      </c>
+      <c r="O9" s="5">
+        <v>116</v>
+      </c>
+      <c r="P9" s="5">
+        <v>35</v>
+      </c>
+      <c r="AA9">
+        <f>LOG(B9)</f>
+        <v>3.3725438007590705</v>
+      </c>
+      <c r="AB9">
+        <f>LOG(C9)</f>
+        <v>4.672734971642158</v>
+      </c>
+      <c r="AC9">
+        <f>LOG(D9)</f>
+        <v>4.8429273560990236</v>
+      </c>
+      <c r="AF9">
+        <f>LOG(E9)</f>
+        <v>2.0791812460476247</v>
+      </c>
+      <c r="AG9">
+        <f>LOG(F9)</f>
+        <v>2.357934847000454</v>
+      </c>
+      <c r="AH9">
+        <f>LOG(G9)</f>
+        <v>1.7923916894982539</v>
+      </c>
+      <c r="AK9">
+        <f>LOG(H9)</f>
+        <v>1.7781512503836436</v>
+      </c>
+      <c r="AL9">
+        <f>LOG(I9)</f>
+        <v>2.0606978403536118</v>
+      </c>
+      <c r="AM9">
+        <f>LOG(J9)</f>
+        <v>0.95424250943932487</v>
+      </c>
+      <c r="AP9">
+        <f t="shared" si="2"/>
+        <v>2.1303337684950061</v>
+      </c>
+      <c r="AQ9">
+        <f t="shared" si="0"/>
+        <v>2.255272505103306</v>
+      </c>
+      <c r="AR9">
+        <f t="shared" si="0"/>
+        <v>1.4313637641589874</v>
+      </c>
+      <c r="AU9">
+        <f t="shared" si="3"/>
+        <v>1.7923916894982539</v>
+      </c>
+      <c r="AV9">
+        <f t="shared" si="1"/>
+        <v>2.0644579892269186</v>
+      </c>
+      <c r="AW9">
+        <f t="shared" si="1"/>
+        <v>1.5440680443502757</v>
+      </c>
+    </row>
+    <row r="10" spans="1:49" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>10</v>
+      </c>
+      <c r="B10" s="1">
+        <v>3468</v>
+      </c>
+      <c r="C10" s="1">
+        <v>75149</v>
+      </c>
+      <c r="D10" s="1">
+        <v>112761</v>
+      </c>
+      <c r="E10" s="2">
+        <v>134</v>
+      </c>
+      <c r="F10" s="2">
+        <v>259</v>
+      </c>
+      <c r="G10" s="2">
+        <v>74</v>
+      </c>
+      <c r="H10" s="3">
+        <v>67</v>
+      </c>
+      <c r="I10" s="3">
+        <v>128</v>
+      </c>
+      <c r="J10" s="3">
+        <v>10</v>
+      </c>
+      <c r="K10" s="4">
+        <v>150</v>
+      </c>
+      <c r="L10" s="4">
+        <v>200</v>
+      </c>
+      <c r="M10" s="4">
+        <v>30</v>
+      </c>
+      <c r="N10" s="5">
+        <v>69</v>
+      </c>
+      <c r="O10" s="5">
+        <v>129</v>
+      </c>
+      <c r="P10" s="5">
+        <v>39</v>
+      </c>
+      <c r="AA10">
+        <f>LOG(B10)</f>
+        <v>3.5400790888041729</v>
+      </c>
+      <c r="AB10">
+        <f>LOG(C10)</f>
+        <v>4.875923205849455</v>
+      </c>
+      <c r="AC10">
+        <f>LOG(D10)</f>
+        <v>5.0521589186766507</v>
+      </c>
+      <c r="AF10">
+        <f>LOG(E10)</f>
+        <v>2.1271047983648077</v>
+      </c>
+      <c r="AG10">
+        <f>LOG(F10)</f>
+        <v>2.4132997640812519</v>
+      </c>
+      <c r="AH10">
+        <f>LOG(G10)</f>
+        <v>1.8692317197309762</v>
+      </c>
+      <c r="AK10">
+        <f>LOG(H10)</f>
+        <v>1.8260748027008264</v>
+      </c>
+      <c r="AL10">
+        <f>LOG(I10)</f>
+        <v>2.1072099696478683</v>
+      </c>
+      <c r="AM10">
+        <f>LOG(J10)</f>
+        <v>1</v>
+      </c>
+      <c r="AP10">
+        <f t="shared" si="2"/>
+        <v>2.1760912590556813</v>
+      </c>
+      <c r="AQ10">
+        <f t="shared" si="0"/>
+        <v>2.3010299956639813</v>
+      </c>
+      <c r="AR10">
+        <f t="shared" si="0"/>
+        <v>1.4771212547196624</v>
+      </c>
+      <c r="AU10">
+        <f t="shared" si="3"/>
+        <v>1.8388490907372552</v>
+      </c>
+      <c r="AV10">
+        <f t="shared" si="1"/>
+        <v>2.1105897102992488</v>
+      </c>
+      <c r="AW10">
+        <f t="shared" si="1"/>
+        <v>1.5910646070264991</v>
+      </c>
+    </row>
+    <row r="11" spans="1:49" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>11</v>
+      </c>
+      <c r="B11" s="1">
+        <v>4931</v>
+      </c>
+      <c r="C11" s="1">
+        <v>115178</v>
+      </c>
+      <c r="D11" s="1">
+        <v>174966</v>
+      </c>
+      <c r="E11" s="2">
+        <v>148</v>
+      </c>
+      <c r="F11" s="2">
+        <v>291</v>
+      </c>
+      <c r="G11" s="2">
+        <v>87</v>
+      </c>
+      <c r="H11" s="3">
+        <v>74</v>
+      </c>
+      <c r="I11" s="3">
+        <v>141</v>
+      </c>
+      <c r="J11" s="3">
+        <v>11</v>
+      </c>
+      <c r="K11" s="4">
+        <v>165</v>
+      </c>
+      <c r="L11" s="4">
+        <v>220</v>
+      </c>
+      <c r="M11" s="4">
+        <v>33</v>
+      </c>
+      <c r="N11" s="5">
+        <v>76</v>
+      </c>
+      <c r="O11" s="5">
+        <v>142</v>
+      </c>
+      <c r="P11" s="5">
+        <v>43</v>
+      </c>
+      <c r="AA11">
+        <f>LOG(B11)</f>
+        <v>3.6929350025311378</v>
+      </c>
+      <c r="AB11">
+        <f>LOG(C11)</f>
+        <v>5.0613695329844326</v>
+      </c>
+      <c r="AC11">
+        <f>LOG(D11)</f>
+        <v>5.242953663274962</v>
+      </c>
+      <c r="AF11">
+        <f>LOG(E11)</f>
+        <v>2.1702617153949575</v>
+      </c>
+      <c r="AG11">
+        <f>LOG(F11)</f>
+        <v>2.4638929889859074</v>
+      </c>
+      <c r="AH11">
+        <f>LOG(G11)</f>
+        <v>1.9395192526186185</v>
+      </c>
+      <c r="AK11">
+        <f>LOG(H11)</f>
+        <v>1.8692317197309762</v>
+      </c>
+      <c r="AL11">
+        <f>LOG(I11)</f>
+        <v>2.1492191126553797</v>
+      </c>
+      <c r="AM11">
+        <f>LOG(J11)</f>
+        <v>1.0413926851582251</v>
+      </c>
+      <c r="AP11">
+        <f t="shared" si="2"/>
+        <v>2.2174839442139063</v>
+      </c>
+      <c r="AQ11">
+        <f t="shared" si="0"/>
+        <v>2.3424226808222062</v>
+      </c>
+      <c r="AR11">
+        <f t="shared" si="0"/>
+        <v>1.5185139398778875</v>
+      </c>
+      <c r="AU11">
+        <f t="shared" si="3"/>
+        <v>1.8808135922807914</v>
+      </c>
+      <c r="AV11">
+        <f t="shared" si="1"/>
+        <v>2.1522883443830563</v>
+      </c>
+      <c r="AW11">
+        <f t="shared" si="1"/>
+        <v>1.6334684555795864</v>
+      </c>
+    </row>
+    <row r="12" spans="1:49" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>12</v>
+      </c>
+      <c r="B12" s="1">
+        <v>6815</v>
+      </c>
+      <c r="C12" s="1">
+        <v>170594</v>
+      </c>
+      <c r="D12" s="1">
+        <v>262002</v>
+      </c>
+      <c r="E12" s="2">
+        <v>162</v>
+      </c>
+      <c r="F12" s="2">
+        <v>324</v>
+      </c>
+      <c r="G12" s="2">
+        <v>101</v>
+      </c>
+      <c r="H12" s="3">
+        <v>81</v>
+      </c>
+      <c r="I12" s="3">
+        <v>154</v>
+      </c>
+      <c r="J12" s="3">
+        <v>12</v>
+      </c>
+      <c r="K12" s="4">
+        <v>180</v>
+      </c>
+      <c r="L12" s="4">
+        <v>240</v>
+      </c>
+      <c r="M12" s="4">
+        <v>36</v>
+      </c>
+      <c r="N12" s="5">
+        <v>83</v>
+      </c>
+      <c r="O12" s="5">
+        <v>155</v>
+      </c>
+      <c r="P12" s="5">
+        <v>47</v>
+      </c>
+      <c r="AA12">
+        <f>LOG(B12)</f>
+        <v>3.8334658601706924</v>
+      </c>
+      <c r="AB12">
+        <f>LOG(C12)</f>
+        <v>5.2319637524310654</v>
+      </c>
+      <c r="AC12">
+        <f>LOG(D12)</f>
+        <v>5.4183046065321445</v>
+      </c>
+      <c r="AF12">
+        <f>LOG(E12)</f>
+        <v>2.2095150145426308</v>
+      </c>
+      <c r="AG12">
+        <f>LOG(F12)</f>
+        <v>2.510545010206612</v>
+      </c>
+      <c r="AH12">
+        <f>LOG(G12)</f>
+        <v>2.0043213737826426</v>
+      </c>
+      <c r="AK12">
+        <f>LOG(H12)</f>
+        <v>1.9084850188786497</v>
+      </c>
+      <c r="AL12">
+        <f>LOG(I12)</f>
+        <v>2.1875207208364631</v>
+      </c>
+      <c r="AM12">
+        <f>LOG(J12)</f>
+        <v>1.0791812460476249</v>
+      </c>
+      <c r="AP12">
+        <f t="shared" si="2"/>
+        <v>2.255272505103306</v>
+      </c>
+      <c r="AQ12">
+        <f t="shared" si="0"/>
+        <v>2.3802112417116059</v>
+      </c>
+      <c r="AR12">
+        <f t="shared" si="0"/>
         <v>1.5563025007672873</v>
       </c>
-      <c r="S3">
+      <c r="AU12">
+        <f t="shared" si="3"/>
+        <v>1.919078092376074</v>
+      </c>
+      <c r="AV12">
+        <f t="shared" si="1"/>
+        <v>2.1903316981702914</v>
+      </c>
+      <c r="AW12">
+        <f t="shared" si="1"/>
+        <v>1.6720978579357175</v>
+      </c>
+    </row>
+    <row r="13" spans="1:49" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>13</v>
+      </c>
+      <c r="B13" s="1">
+        <v>9194</v>
+      </c>
+      <c r="C13" s="1">
+        <v>245435</v>
+      </c>
+      <c r="D13" s="1">
+        <v>380653</v>
+      </c>
+      <c r="E13" s="2">
+        <v>176</v>
+      </c>
+      <c r="F13" s="2">
+        <v>358</v>
+      </c>
+      <c r="G13" s="2">
+        <v>116</v>
+      </c>
+      <c r="H13" s="3">
+        <v>88</v>
+      </c>
+      <c r="I13" s="3">
+        <v>167</v>
+      </c>
+      <c r="J13" s="3">
+        <v>13</v>
+      </c>
+      <c r="K13" s="4">
+        <v>195</v>
+      </c>
+      <c r="L13" s="4">
+        <v>260</v>
+      </c>
+      <c r="M13" s="4">
+        <v>39</v>
+      </c>
+      <c r="N13" s="5">
+        <v>90</v>
+      </c>
+      <c r="O13" s="5">
+        <v>168</v>
+      </c>
+      <c r="P13" s="5">
+        <v>51</v>
+      </c>
+      <c r="AA13">
+        <f>LOG(B13)</f>
+        <v>3.9635044994142907</v>
+      </c>
+      <c r="AB13">
+        <f>LOG(C13)</f>
+        <v>5.389936494915041</v>
+      </c>
+      <c r="AC13">
+        <f>LOG(D13)</f>
+        <v>5.5805292569017242</v>
+      </c>
+      <c r="AF13">
+        <f>LOG(E13)</f>
+        <v>2.2455126678141499</v>
+      </c>
+      <c r="AG13">
+        <f>LOG(F13)</f>
+        <v>2.5538830266438746</v>
+      </c>
+      <c r="AH13">
+        <f>LOG(G13)</f>
+        <v>2.0644579892269186</v>
+      </c>
+      <c r="AK13">
+        <f>LOG(H13)</f>
+        <v>1.9444826721501687</v>
+      </c>
+      <c r="AL13">
+        <f>LOG(I13)</f>
+        <v>2.2227164711475833</v>
+      </c>
+      <c r="AM13">
+        <f>LOG(J13)</f>
+        <v>1.1139433523068367</v>
+      </c>
+      <c r="AP13">
+        <f t="shared" si="2"/>
+        <v>2.2900346113625178</v>
+      </c>
+      <c r="AQ13">
+        <f t="shared" si="0"/>
+        <v>2.4149733479708178</v>
+      </c>
+      <c r="AR13">
+        <f t="shared" si="0"/>
+        <v>1.5910646070264991</v>
+      </c>
+      <c r="AU13">
+        <f t="shared" si="3"/>
+        <v>1.954242509439325</v>
+      </c>
+      <c r="AV13">
+        <f t="shared" si="1"/>
+        <v>2.2253092817258628</v>
+      </c>
+      <c r="AW13">
+        <f t="shared" si="1"/>
+        <v>1.7075701760979363</v>
+      </c>
+    </row>
+    <row r="14" spans="1:49" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>14</v>
+      </c>
+      <c r="B14" s="1">
+        <v>12148</v>
+      </c>
+      <c r="C14" s="1">
+        <v>344387</v>
+      </c>
+      <c r="D14" s="1">
+        <v>538839</v>
+      </c>
+      <c r="E14" s="2">
+        <v>190</v>
+      </c>
+      <c r="F14" s="2">
+        <v>393</v>
+      </c>
+      <c r="G14" s="2">
+        <v>132</v>
+      </c>
+      <c r="H14" s="3">
+        <v>95</v>
+      </c>
+      <c r="I14" s="3">
+        <v>180</v>
+      </c>
+      <c r="J14" s="3">
+        <v>14</v>
+      </c>
+      <c r="K14" s="4">
+        <v>210</v>
+      </c>
+      <c r="L14" s="4">
+        <v>280</v>
+      </c>
+      <c r="M14" s="4">
+        <v>42</v>
+      </c>
+      <c r="N14" s="5">
+        <v>97</v>
+      </c>
+      <c r="O14" s="5">
+        <v>181</v>
+      </c>
+      <c r="P14" s="5">
+        <v>55</v>
+      </c>
+      <c r="AA14">
+        <f>LOG(B14)</f>
+        <v>4.0845047832462278</v>
+      </c>
+      <c r="AB14">
+        <f>LOG(C14)</f>
+        <v>5.5370467492426405</v>
+      </c>
+      <c r="AC14">
+        <f>LOG(D14)</f>
+        <v>5.7314590214827037</v>
+      </c>
+      <c r="AF14">
+        <f>LOG(E14)</f>
+        <v>2.2787536009528289</v>
+      </c>
+      <c r="AG14">
+        <f>LOG(F14)</f>
+        <v>2.5943925503754266</v>
+      </c>
+      <c r="AH14">
+        <f>LOG(G14)</f>
+        <v>2.12057393120585</v>
+      </c>
+      <c r="AK14">
+        <f>LOG(H14)</f>
+        <v>1.9777236052888478</v>
+      </c>
+      <c r="AL14">
+        <f>LOG(I14)</f>
+        <v>2.255272505103306</v>
+      </c>
+      <c r="AM14">
+        <f>LOG(J14)</f>
+        <v>1.146128035678238</v>
+      </c>
+      <c r="AP14">
+        <f t="shared" si="2"/>
+        <v>2.3222192947339191</v>
+      </c>
+      <c r="AQ14">
+        <f t="shared" si="0"/>
+        <v>2.4471580313422194</v>
+      </c>
+      <c r="AR14">
+        <f t="shared" si="0"/>
+        <v>1.6232492903979006</v>
+      </c>
+      <c r="AU14">
+        <f t="shared" si="3"/>
+        <v>1.9867717342662448</v>
+      </c>
+      <c r="AV14">
+        <f t="shared" si="1"/>
+        <v>2.2576785748691846</v>
+      </c>
+      <c r="AW14">
+        <f t="shared" si="1"/>
+        <v>1.7403626894942439</v>
+      </c>
+    </row>
+    <row r="15" spans="1:49" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>15</v>
+      </c>
+      <c r="B15" s="1">
+        <v>15763</v>
+      </c>
+      <c r="C15" s="1">
+        <v>472832</v>
+      </c>
+      <c r="D15" s="1">
+        <v>745704</v>
+      </c>
+      <c r="E15" s="2">
+        <v>204</v>
+      </c>
+      <c r="F15" s="2">
+        <v>429</v>
+      </c>
+      <c r="G15" s="2">
+        <v>149</v>
+      </c>
+      <c r="H15" s="3">
+        <v>102</v>
+      </c>
+      <c r="I15" s="3">
+        <v>193</v>
+      </c>
+      <c r="J15" s="3">
+        <v>15</v>
+      </c>
+      <c r="K15" s="4">
+        <v>225</v>
+      </c>
+      <c r="L15" s="4">
+        <v>300</v>
+      </c>
+      <c r="M15" s="4">
+        <v>45</v>
+      </c>
+      <c r="N15" s="5">
+        <v>104</v>
+      </c>
+      <c r="O15" s="5">
+        <v>194</v>
+      </c>
+      <c r="P15" s="5">
+        <v>59</v>
+      </c>
+      <c r="AA15">
+        <f>LOG(B15)</f>
+        <v>4.1976388755555698</v>
+      </c>
+      <c r="AB15">
+        <f>LOG(C15)</f>
+        <v>5.6747068607520914</v>
+      </c>
+      <c r="AC15">
+        <f>LOG(D15)</f>
+        <v>5.8725664726779767</v>
+      </c>
+      <c r="AF15">
+        <f>LOG(E15)</f>
+        <v>2.3096301674258988</v>
+      </c>
+      <c r="AG15">
+        <f>LOG(F15)</f>
+        <v>2.6324572921847245</v>
+      </c>
+      <c r="AH15">
+        <f>LOG(G15)</f>
+        <v>2.173186268412274</v>
+      </c>
+      <c r="AK15">
+        <f>LOG(H15)</f>
+        <v>2.0086001717619175</v>
+      </c>
+      <c r="AL15">
+        <f>LOG(I15)</f>
+        <v>2.2855573090077739</v>
+      </c>
+      <c r="AM15">
+        <f>LOG(J15)</f>
+        <v>1.1760912590556813</v>
+      </c>
+      <c r="AP15">
+        <f t="shared" si="2"/>
+        <v>2.3521825181113627</v>
+      </c>
+      <c r="AQ15">
+        <f t="shared" si="0"/>
+        <v>2.4771212547196626</v>
+      </c>
+      <c r="AR15">
+        <f t="shared" si="0"/>
+        <v>1.6532125137753437</v>
+      </c>
+      <c r="AU15">
+        <f t="shared" si="3"/>
+        <v>2.0170333392987803</v>
+      </c>
+      <c r="AV15">
+        <f t="shared" si="1"/>
+        <v>2.287801729930226</v>
+      </c>
+      <c r="AW15">
+        <f t="shared" si="1"/>
+        <v>1.7708520116421442</v>
+      </c>
+    </row>
+    <row r="16" spans="1:49" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>16</v>
+      </c>
+      <c r="B16" s="1">
+        <v>20131</v>
+      </c>
+      <c r="C16" s="1">
+        <v>636896</v>
+      </c>
+      <c r="D16" s="1">
+        <v>1011704</v>
+      </c>
+      <c r="E16" s="2">
+        <v>218</v>
+      </c>
+      <c r="F16" s="2">
+        <v>466</v>
+      </c>
+      <c r="G16" s="2">
+        <v>167</v>
+      </c>
+      <c r="H16" s="3">
+        <v>109</v>
+      </c>
+      <c r="I16" s="3">
+        <v>206</v>
+      </c>
+      <c r="J16" s="3">
+        <v>16</v>
+      </c>
+      <c r="K16" s="4">
+        <v>240</v>
+      </c>
+      <c r="L16" s="4">
+        <v>320</v>
+      </c>
+      <c r="M16" s="4">
+        <v>48</v>
+      </c>
+      <c r="N16" s="5">
+        <v>111</v>
+      </c>
+      <c r="O16" s="5">
+        <v>207</v>
+      </c>
+      <c r="P16" s="5">
+        <v>63</v>
+      </c>
+      <c r="AA16">
+        <f>LOG(B16)</f>
+        <v>4.3038653488427041</v>
+      </c>
+      <c r="AB16">
+        <f>LOG(C16)</f>
+        <v>5.8040685213250036</v>
+      </c>
+      <c r="AC16">
+        <f>LOG(D16)</f>
+        <v>6.0050534670785991</v>
+      </c>
+      <c r="AF16">
+        <f>LOG(E16)</f>
+        <v>2.3384564936046046</v>
+      </c>
+      <c r="AG16">
+        <f>LOG(F16)</f>
+        <v>2.6683859166900001</v>
+      </c>
+      <c r="AH16">
+        <f>LOG(G16)</f>
+        <v>2.2227164711475833</v>
+      </c>
+      <c r="AK16">
+        <f>LOG(H16)</f>
+        <v>2.0374264979406238</v>
+      </c>
+      <c r="AL16">
+        <f>LOG(I16)</f>
+        <v>2.3138672203691533</v>
+      </c>
+      <c r="AM16">
+        <f>LOG(J16)</f>
+        <v>1.2041199826559248</v>
+      </c>
+      <c r="AP16">
+        <f t="shared" si="2"/>
+        <v>2.3802112417116059</v>
+      </c>
+      <c r="AQ16">
+        <f t="shared" si="0"/>
+        <v>2.5051499783199058</v>
+      </c>
+      <c r="AR16">
+        <f t="shared" si="0"/>
+        <v>1.6812412373755872</v>
+      </c>
+      <c r="AU16">
+        <f t="shared" si="3"/>
+        <v>2.0453229787866576</v>
+      </c>
+      <c r="AV16">
+        <f t="shared" si="1"/>
+        <v>2.3159703454569178</v>
+      </c>
+      <c r="AW16">
         <f t="shared" si="1"/>
         <v>1.7993405494535817</v>
       </c>
-      <c r="T3">
+    </row>
+    <row r="17" spans="1:49" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>17</v>
+      </c>
+      <c r="B17" s="1">
+        <v>25350</v>
+      </c>
+      <c r="C17" s="1">
+        <v>843497</v>
+      </c>
+      <c r="D17" s="1">
+        <v>1348695</v>
+      </c>
+      <c r="E17" s="2">
+        <v>232</v>
+      </c>
+      <c r="F17" s="2">
+        <v>504</v>
+      </c>
+      <c r="G17" s="2">
+        <v>186</v>
+      </c>
+      <c r="H17" s="3">
+        <v>116</v>
+      </c>
+      <c r="I17" s="3">
+        <v>219</v>
+      </c>
+      <c r="J17" s="3">
+        <v>17</v>
+      </c>
+      <c r="K17" s="4">
+        <v>255</v>
+      </c>
+      <c r="L17" s="4">
+        <v>340</v>
+      </c>
+      <c r="M17" s="4">
+        <v>51</v>
+      </c>
+      <c r="N17" s="5">
+        <v>118</v>
+      </c>
+      <c r="O17" s="5">
+        <v>220</v>
+      </c>
+      <c r="P17" s="5">
+        <v>67</v>
+      </c>
+      <c r="AA17">
+        <f>LOG(B17)</f>
+        <v>4.4039779636693543</v>
+      </c>
+      <c r="AB17">
+        <f>LOG(C17)</f>
+        <v>5.926083542306575</v>
+      </c>
+      <c r="AC17">
+        <f>LOG(D17)</f>
+        <v>6.1299137474529397</v>
+      </c>
+      <c r="AF17">
+        <f>LOG(E17)</f>
+        <v>2.3654879848908998</v>
+      </c>
+      <c r="AG17">
+        <f>LOG(F17)</f>
+        <v>2.7024305364455254</v>
+      </c>
+      <c r="AH17">
+        <f>LOG(G17)</f>
+        <v>2.2695129442179165</v>
+      </c>
+      <c r="AK17">
+        <f>LOG(H17)</f>
+        <v>2.0644579892269186</v>
+      </c>
+      <c r="AL17">
+        <f>LOG(I17)</f>
+        <v>2.3404441148401185</v>
+      </c>
+      <c r="AM17">
+        <f>LOG(J17)</f>
+        <v>1.2304489213782739</v>
+      </c>
+      <c r="AP17">
+        <f t="shared" si="2"/>
+        <v>2.406540180433955</v>
+      </c>
+      <c r="AQ17">
+        <f t="shared" si="0"/>
+        <v>2.5314789170422549</v>
+      </c>
+      <c r="AR17">
+        <f t="shared" si="0"/>
+        <v>1.7075701760979363</v>
+      </c>
+      <c r="AU17">
+        <f t="shared" si="3"/>
+        <v>2.0718820073061255</v>
+      </c>
+      <c r="AV17">
         <f t="shared" si="1"/>
-        <v>1.0413926851582251</v>
-      </c>
-      <c r="W3">
-        <f t="shared" ref="W3:W20" si="5">LOG(H3)</f>
+        <v>2.3424226808222062</v>
+      </c>
+      <c r="AW17">
+        <f t="shared" si="1"/>
+        <v>1.8260748027008264</v>
+      </c>
+    </row>
+    <row r="18" spans="1:49" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>18</v>
+      </c>
+      <c r="B18" s="1">
+        <v>31524</v>
+      </c>
+      <c r="C18" s="1">
+        <v>1100393</v>
+      </c>
+      <c r="D18" s="1">
+        <v>1770021</v>
+      </c>
+      <c r="E18" s="2">
+        <v>246</v>
+      </c>
+      <c r="F18" s="2">
+        <v>543</v>
+      </c>
+      <c r="G18" s="2">
+        <v>206</v>
+      </c>
+      <c r="H18" s="3">
+        <v>123</v>
+      </c>
+      <c r="I18" s="3">
+        <v>232</v>
+      </c>
+      <c r="J18" s="3">
+        <v>18</v>
+      </c>
+      <c r="K18" s="4">
+        <v>270</v>
+      </c>
+      <c r="L18" s="4">
+        <v>360</v>
+      </c>
+      <c r="M18" s="4">
+        <v>54</v>
+      </c>
+      <c r="N18" s="5">
+        <v>125</v>
+      </c>
+      <c r="O18" s="5">
+        <v>233</v>
+      </c>
+      <c r="P18" s="5">
+        <v>71</v>
+      </c>
+      <c r="AA18">
+        <f>LOG(B18)</f>
+        <v>4.4986413188336947</v>
+      </c>
+      <c r="AB18">
+        <f>LOG(C18)</f>
+        <v>6.0415478190213152</v>
+      </c>
+      <c r="AC18">
+        <f>LOG(D18)</f>
+        <v>6.2479784189776355</v>
+      </c>
+      <c r="AF18">
+        <f>LOG(E18)</f>
+        <v>2.3909351071033793</v>
+      </c>
+      <c r="AG18">
+        <f>LOG(F18)</f>
+        <v>2.7347998295888472</v>
+      </c>
+      <c r="AH18">
+        <f>LOG(G18)</f>
+        <v>2.3138672203691533</v>
+      </c>
+      <c r="AK18">
+        <f>LOG(H18)</f>
+        <v>2.0899051114393981</v>
+      </c>
+      <c r="AL18">
+        <f>LOG(I18)</f>
+        <v>2.3654879848908998</v>
+      </c>
+      <c r="AM18">
+        <f>LOG(J18)</f>
         <v>1.255272505103306</v>
       </c>
-      <c r="X3">
+      <c r="AP18">
         <f t="shared" si="2"/>
-        <v>1.568201724066995</v>
-      </c>
-      <c r="Y3">
+        <v>2.4313637641589874</v>
+      </c>
+      <c r="AQ18">
+        <f t="shared" ref="AQ18:AQ20" si="4">LOG(L18)</f>
+        <v>2.5563025007672873</v>
+      </c>
+      <c r="AR18">
+        <f t="shared" ref="AR18:AR20" si="5">LOG(M18)</f>
+        <v>1.7323937598229686</v>
+      </c>
+      <c r="AU18">
+        <f t="shared" si="3"/>
+        <v>2.0969100130080562</v>
+      </c>
+      <c r="AV18">
+        <f t="shared" ref="AV18:AV20" si="6">LOG(O18)</f>
+        <v>2.3673559210260189</v>
+      </c>
+      <c r="AW18">
+        <f t="shared" ref="AW18:AW20" si="7">LOG(P18)</f>
+        <v>1.8512583487190752</v>
+      </c>
+    </row>
+    <row r="19" spans="1:49" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>19</v>
+      </c>
+      <c r="B19" s="1">
+        <v>38763</v>
+      </c>
+      <c r="C19" s="1">
+        <v>1416230</v>
+      </c>
+      <c r="D19" s="1">
+        <v>2290602</v>
+      </c>
+      <c r="E19" s="2">
+        <v>260</v>
+      </c>
+      <c r="F19" s="2">
+        <v>583</v>
+      </c>
+      <c r="G19" s="2">
+        <v>227</v>
+      </c>
+      <c r="H19" s="3">
+        <v>130</v>
+      </c>
+      <c r="I19" s="3">
+        <v>245</v>
+      </c>
+      <c r="J19" s="3">
+        <v>19</v>
+      </c>
+      <c r="K19" s="4">
+        <v>285</v>
+      </c>
+      <c r="L19" s="4">
+        <v>380</v>
+      </c>
+      <c r="M19" s="4">
+        <v>57</v>
+      </c>
+      <c r="N19" s="5">
+        <v>132</v>
+      </c>
+      <c r="O19" s="5">
+        <v>246</v>
+      </c>
+      <c r="P19" s="5">
+        <v>75</v>
+      </c>
+      <c r="AA19">
+        <f>LOG(B19)</f>
+        <v>4.5884173812019249</v>
+      </c>
+      <c r="AB19">
+        <f>LOG(C19)</f>
+        <v>6.151133789808104</v>
+      </c>
+      <c r="AC19">
+        <f>LOG(D19)</f>
+        <v>6.3599496355798379</v>
+      </c>
+      <c r="AF19">
+        <f>LOG(E19)</f>
+        <v>2.4149733479708178</v>
+      </c>
+      <c r="AG19">
+        <f>LOG(F19)</f>
+        <v>2.7656685547590141</v>
+      </c>
+      <c r="AH19">
+        <f>LOG(G19)</f>
+        <v>2.3560258571931225</v>
+      </c>
+      <c r="AK19">
+        <f>LOG(H19)</f>
+        <v>2.1139433523068369</v>
+      </c>
+      <c r="AL19">
+        <f>LOG(I19)</f>
+        <v>2.3891660843645326</v>
+      </c>
+      <c r="AM19">
+        <f>LOG(J19)</f>
+        <v>1.2787536009528289</v>
+      </c>
+      <c r="AP19">
         <f t="shared" si="2"/>
-        <v>0.47712125471966244</v>
+        <v>2.4548448600085102</v>
+      </c>
+      <c r="AQ19">
+        <f t="shared" si="4"/>
+        <v>2.5797835966168101</v>
+      </c>
+      <c r="AR19">
+        <f t="shared" si="5"/>
+        <v>1.7558748556724915</v>
+      </c>
+      <c r="AU19">
+        <f t="shared" si="3"/>
+        <v>2.12057393120585</v>
+      </c>
+      <c r="AV19">
+        <f t="shared" si="6"/>
+        <v>2.3909351071033793</v>
+      </c>
+      <c r="AW19">
+        <f t="shared" si="7"/>
+        <v>1.8750612633917001</v>
       </c>
     </row>
-    <row r="4" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A4">
-        <v>4</v>
-      </c>
-      <c r="B4">
-        <v>143</v>
-      </c>
-      <c r="C4">
-        <v>1526</v>
-      </c>
-      <c r="D4">
-        <v>2038</v>
-      </c>
-      <c r="E4">
-        <v>50</v>
-      </c>
-      <c r="F4">
-        <v>88</v>
-      </c>
-      <c r="G4">
-        <v>17</v>
-      </c>
-      <c r="H4">
-        <v>25</v>
-      </c>
-      <c r="I4">
-        <v>50</v>
-      </c>
-      <c r="J4">
-        <v>4</v>
-      </c>
-      <c r="M4">
-        <f t="shared" si="3"/>
-        <v>2.1553360374650619</v>
-      </c>
-      <c r="N4">
-        <f t="shared" si="0"/>
-        <v>3.1835545336188615</v>
-      </c>
-      <c r="O4">
-        <f t="shared" si="0"/>
-        <v>3.3092041796704077</v>
-      </c>
-      <c r="R4">
+    <row r="20" spans="1:49" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>20</v>
+      </c>
+      <c r="B20" s="1">
+        <v>47183</v>
+      </c>
+      <c r="C20" s="1">
+        <v>1800590</v>
+      </c>
+      <c r="D20" s="1">
+        <v>2927022</v>
+      </c>
+      <c r="E20" s="2">
+        <v>274</v>
+      </c>
+      <c r="F20" s="2">
+        <v>624</v>
+      </c>
+      <c r="G20" s="2">
+        <v>249</v>
+      </c>
+      <c r="H20" s="3">
+        <v>137</v>
+      </c>
+      <c r="I20" s="3">
+        <v>258</v>
+      </c>
+      <c r="J20" s="3">
+        <v>20</v>
+      </c>
+      <c r="K20" s="4">
+        <v>300</v>
+      </c>
+      <c r="L20" s="4">
+        <v>400</v>
+      </c>
+      <c r="M20" s="4">
+        <v>60</v>
+      </c>
+      <c r="N20" s="5">
+        <v>139</v>
+      </c>
+      <c r="O20" s="5">
+        <v>259</v>
+      </c>
+      <c r="P20" s="5">
+        <v>79</v>
+      </c>
+      <c r="AA20">
+        <f>LOG(B20)</f>
+        <v>4.6737855508358148</v>
+      </c>
+      <c r="AB20">
+        <f>LOG(C20)</f>
+        <v>6.2554148338586577</v>
+      </c>
+      <c r="AC20">
+        <f>LOG(D20)</f>
+        <v>6.4664259866779652</v>
+      </c>
+      <c r="AF20">
+        <f>LOG(E20)</f>
+        <v>2.4377505628203879</v>
+      </c>
+      <c r="AG20">
+        <f>LOG(F20)</f>
+        <v>2.7951845896824241</v>
+      </c>
+      <c r="AH20">
+        <f>LOG(G20)</f>
+        <v>2.3961993470957363</v>
+      </c>
+      <c r="AK20">
+        <f>LOG(H20)</f>
+        <v>2.1367205671564067</v>
+      </c>
+      <c r="AL20">
+        <f>LOG(I20)</f>
+        <v>2.4116197059632301</v>
+      </c>
+      <c r="AM20">
+        <f>LOG(J20)</f>
+        <v>1.3010299956639813</v>
+      </c>
+      <c r="AP20">
+        <f t="shared" si="2"/>
+        <v>2.4771212547196626</v>
+      </c>
+      <c r="AQ20">
         <f t="shared" si="4"/>
-        <v>1.6989700043360187</v>
-      </c>
-      <c r="S4">
-        <f t="shared" si="1"/>
-        <v>1.9444826721501687</v>
-      </c>
-      <c r="T4">
-        <f t="shared" si="1"/>
-        <v>1.2304489213782739</v>
-      </c>
-      <c r="W4">
-        <f t="shared" si="5"/>
-        <v>1.3979400086720377</v>
-      </c>
-      <c r="X4">
-        <f t="shared" si="2"/>
-        <v>1.6989700043360187</v>
-      </c>
-      <c r="Y4">
-        <f t="shared" si="2"/>
-        <v>0.6020599913279624</v>
-      </c>
-    </row>
-    <row r="5" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A5">
-        <v>5</v>
-      </c>
-      <c r="B5">
-        <v>298</v>
-      </c>
-      <c r="C5">
-        <v>3791</v>
-      </c>
-      <c r="D5">
-        <v>5193</v>
-      </c>
-      <c r="E5">
-        <v>64</v>
-      </c>
-      <c r="F5">
-        <v>114</v>
-      </c>
-      <c r="G5">
-        <v>24</v>
-      </c>
-      <c r="H5">
-        <v>32</v>
-      </c>
-      <c r="I5">
-        <v>63</v>
-      </c>
-      <c r="J5">
-        <v>5</v>
-      </c>
-      <c r="M5">
-        <f t="shared" si="3"/>
-        <v>2.4742162640762553</v>
-      </c>
-      <c r="N5">
-        <f t="shared" si="0"/>
-        <v>3.5787537844264348</v>
-      </c>
-      <c r="O5">
-        <f t="shared" si="0"/>
-        <v>3.7154183225950561</v>
-      </c>
-      <c r="R5">
-        <f t="shared" si="4"/>
-        <v>1.8061799739838871</v>
-      </c>
-      <c r="S5">
-        <f t="shared" si="1"/>
-        <v>2.0569048513364727</v>
-      </c>
-      <c r="T5">
-        <f t="shared" si="1"/>
-        <v>1.3802112417116059</v>
-      </c>
-      <c r="W5">
-        <f t="shared" si="5"/>
-        <v>1.505149978319906</v>
-      </c>
-      <c r="X5">
-        <f t="shared" si="2"/>
-        <v>1.7993405494535817</v>
-      </c>
-      <c r="Y5">
-        <f t="shared" si="2"/>
-        <v>0.69897000433601886</v>
-      </c>
-    </row>
-    <row r="6" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A6">
-        <v>6</v>
-      </c>
-      <c r="B6">
-        <v>556</v>
-      </c>
-      <c r="C6">
-        <v>8135</v>
-      </c>
-      <c r="D6">
-        <v>11403</v>
-      </c>
-      <c r="E6">
-        <v>78</v>
-      </c>
-      <c r="F6">
-        <v>141</v>
-      </c>
-      <c r="G6">
-        <v>32</v>
-      </c>
-      <c r="H6">
-        <v>39</v>
-      </c>
-      <c r="I6">
-        <v>76</v>
-      </c>
-      <c r="J6">
-        <v>6</v>
-      </c>
-      <c r="M6">
-        <f t="shared" si="3"/>
-        <v>2.7450747915820575</v>
-      </c>
-      <c r="N6">
-        <f t="shared" si="0"/>
-        <v>3.9103575572728775</v>
-      </c>
-      <c r="O6">
-        <f t="shared" si="0"/>
-        <v>4.0570191243227658</v>
-      </c>
-      <c r="R6">
-        <f t="shared" si="4"/>
-        <v>1.8920946026904804</v>
-      </c>
-      <c r="S6">
-        <f t="shared" si="1"/>
-        <v>2.1492191126553797</v>
-      </c>
-      <c r="T6">
-        <f t="shared" si="1"/>
-        <v>1.505149978319906</v>
-      </c>
-      <c r="W6">
-        <f t="shared" si="5"/>
-        <v>1.5910646070264991</v>
-      </c>
-      <c r="X6">
-        <f t="shared" si="2"/>
-        <v>1.8808135922807914</v>
-      </c>
-      <c r="Y6">
-        <f t="shared" si="2"/>
-        <v>0.77815125038364363</v>
-      </c>
-    </row>
-    <row r="7" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A7">
-        <v>7</v>
-      </c>
-      <c r="B7">
-        <v>955</v>
-      </c>
-      <c r="C7">
-        <v>15716</v>
-      </c>
-      <c r="D7">
-        <v>22484</v>
-      </c>
-      <c r="E7">
-        <v>92</v>
-      </c>
-      <c r="F7">
-        <v>169</v>
-      </c>
-      <c r="G7">
-        <v>41</v>
-      </c>
-      <c r="H7">
-        <v>46</v>
-      </c>
-      <c r="I7">
-        <v>89</v>
-      </c>
-      <c r="J7">
-        <v>7</v>
-      </c>
-      <c r="M7">
-        <f t="shared" si="3"/>
-        <v>2.9800033715837464</v>
-      </c>
-      <c r="N7">
-        <f t="shared" si="0"/>
-        <v>4.1963420201397685</v>
-      </c>
-      <c r="O7">
-        <f t="shared" si="0"/>
-        <v>4.3518735766208998</v>
-      </c>
-      <c r="R7">
-        <f t="shared" si="4"/>
-        <v>1.9637878273455553</v>
-      </c>
-      <c r="S7">
-        <f t="shared" si="1"/>
-        <v>2.2278867046136734</v>
-      </c>
-      <c r="T7">
-        <f t="shared" si="1"/>
-        <v>1.6127838567197355</v>
-      </c>
-      <c r="W7">
-        <f t="shared" si="5"/>
-        <v>1.6627578316815741</v>
-      </c>
-      <c r="X7">
-        <f t="shared" si="2"/>
-        <v>1.9493900066449128</v>
-      </c>
-      <c r="Y7">
-        <f t="shared" si="2"/>
-        <v>0.84509804001425681</v>
-      </c>
-    </row>
-    <row r="8" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A8">
-        <v>8</v>
-      </c>
-      <c r="B8">
-        <v>1539</v>
-      </c>
-      <c r="C8">
-        <v>28052</v>
-      </c>
-      <c r="D8">
-        <v>40860</v>
-      </c>
-      <c r="E8">
-        <v>106</v>
-      </c>
-      <c r="F8">
-        <v>198</v>
-      </c>
-      <c r="G8">
-        <v>51</v>
-      </c>
-      <c r="H8">
-        <v>53</v>
-      </c>
-      <c r="I8">
-        <v>102</v>
-      </c>
-      <c r="J8">
-        <v>8</v>
-      </c>
-      <c r="M8">
-        <f t="shared" si="3"/>
-        <v>3.1872386198314788</v>
-      </c>
-      <c r="N8">
-        <f t="shared" si="0"/>
-        <v>4.4479638302267448</v>
-      </c>
-      <c r="O8">
-        <f t="shared" si="0"/>
-        <v>4.611298362296429</v>
-      </c>
-      <c r="R8">
-        <f t="shared" si="4"/>
-        <v>2.0253058652647704</v>
-      </c>
-      <c r="S8">
-        <f t="shared" si="1"/>
-        <v>2.2966651902615309</v>
-      </c>
-      <c r="T8">
-        <f t="shared" si="1"/>
-        <v>1.7075701760979363</v>
-      </c>
-      <c r="W8">
-        <f t="shared" si="5"/>
-        <v>1.7242758696007889</v>
-      </c>
-      <c r="X8">
-        <f t="shared" si="2"/>
-        <v>2.0086001717619175</v>
-      </c>
-      <c r="Y8">
-        <f t="shared" si="2"/>
-        <v>0.90308998699194354</v>
-      </c>
-    </row>
-    <row r="9" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A9">
-        <v>9</v>
-      </c>
-      <c r="B9">
-        <v>2358</v>
-      </c>
-      <c r="C9">
-        <v>47069</v>
-      </c>
-      <c r="D9">
-        <v>69651</v>
-      </c>
-      <c r="E9">
-        <v>120</v>
-      </c>
-      <c r="F9">
-        <v>228</v>
-      </c>
-      <c r="G9">
-        <v>62</v>
-      </c>
-      <c r="H9">
-        <v>60</v>
-      </c>
-      <c r="I9">
-        <v>115</v>
-      </c>
-      <c r="J9">
-        <v>9</v>
-      </c>
-      <c r="M9">
-        <f t="shared" si="3"/>
-        <v>3.3725438007590705</v>
-      </c>
-      <c r="N9">
-        <f t="shared" si="0"/>
-        <v>4.672734971642158</v>
-      </c>
-      <c r="O9">
-        <f t="shared" si="0"/>
-        <v>4.8429273560990236</v>
-      </c>
-      <c r="R9">
-        <f t="shared" si="4"/>
-        <v>2.0791812460476247</v>
-      </c>
-      <c r="S9">
-        <f t="shared" si="1"/>
-        <v>2.357934847000454</v>
-      </c>
-      <c r="T9">
-        <f t="shared" si="1"/>
-        <v>1.7923916894982539</v>
-      </c>
-      <c r="W9">
+        <v>2.6020599913279625</v>
+      </c>
+      <c r="AR20">
         <f t="shared" si="5"/>
         <v>1.7781512503836436</v>
       </c>
-      <c r="X9">
-        <f t="shared" si="2"/>
-        <v>2.0606978403536118</v>
-      </c>
-      <c r="Y9">
-        <f t="shared" si="2"/>
-        <v>0.95424250943932487</v>
+      <c r="AU20">
+        <f t="shared" si="3"/>
+        <v>2.143014800254095</v>
+      </c>
+      <c r="AV20">
+        <f t="shared" si="6"/>
+        <v>2.4132997640812519</v>
+      </c>
+      <c r="AW20">
+        <f t="shared" si="7"/>
+        <v>1.8976270912904414</v>
       </c>
     </row>
-    <row r="10" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A10">
-        <v>10</v>
-      </c>
-      <c r="B10">
-        <v>3468</v>
-      </c>
-      <c r="C10">
-        <v>75149</v>
-      </c>
-      <c r="D10">
-        <v>112761</v>
-      </c>
-      <c r="E10">
-        <v>134</v>
-      </c>
-      <c r="F10">
-        <v>259</v>
-      </c>
-      <c r="G10">
-        <v>74</v>
-      </c>
-      <c r="H10">
-        <v>67</v>
-      </c>
-      <c r="I10">
-        <v>128</v>
-      </c>
-      <c r="J10">
-        <v>10</v>
-      </c>
-      <c r="M10">
-        <f t="shared" si="3"/>
-        <v>3.5400790888041729</v>
-      </c>
-      <c r="N10">
-        <f t="shared" si="0"/>
-        <v>4.875923205849455</v>
-      </c>
-      <c r="O10">
-        <f t="shared" si="0"/>
-        <v>5.0521589186766507</v>
-      </c>
-      <c r="R10">
-        <f t="shared" si="4"/>
-        <v>2.1271047983648077</v>
-      </c>
-      <c r="S10">
-        <f t="shared" si="1"/>
-        <v>2.4132997640812519</v>
-      </c>
-      <c r="T10">
-        <f t="shared" si="1"/>
-        <v>1.8692317197309762</v>
-      </c>
-      <c r="W10">
-        <f t="shared" si="5"/>
-        <v>1.8260748027008264</v>
-      </c>
-      <c r="X10">
-        <f t="shared" si="2"/>
-        <v>2.1072099696478683</v>
-      </c>
-      <c r="Y10">
-        <f t="shared" si="2"/>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A11">
-        <v>11</v>
-      </c>
-      <c r="B11">
-        <v>4931</v>
-      </c>
-      <c r="C11">
-        <v>115178</v>
-      </c>
-      <c r="D11">
-        <v>174966</v>
-      </c>
-      <c r="E11">
-        <v>148</v>
-      </c>
-      <c r="F11">
-        <v>291</v>
-      </c>
-      <c r="G11">
-        <v>87</v>
-      </c>
-      <c r="H11">
-        <v>74</v>
-      </c>
-      <c r="I11">
-        <v>141</v>
-      </c>
-      <c r="J11">
-        <v>11</v>
-      </c>
-      <c r="M11">
-        <f t="shared" si="3"/>
-        <v>3.6929350025311378</v>
-      </c>
-      <c r="N11">
-        <f t="shared" si="0"/>
-        <v>5.0613695329844326</v>
-      </c>
-      <c r="O11">
-        <f t="shared" si="0"/>
-        <v>5.242953663274962</v>
-      </c>
-      <c r="R11">
-        <f t="shared" si="4"/>
-        <v>2.1702617153949575</v>
-      </c>
-      <c r="S11">
-        <f t="shared" si="1"/>
-        <v>2.4638929889859074</v>
-      </c>
-      <c r="T11">
-        <f t="shared" si="1"/>
-        <v>1.9395192526186185</v>
-      </c>
-      <c r="W11">
-        <f t="shared" si="5"/>
-        <v>1.8692317197309762</v>
-      </c>
-      <c r="X11">
-        <f t="shared" si="2"/>
-        <v>2.1492191126553797</v>
-      </c>
-      <c r="Y11">
-        <f t="shared" si="2"/>
-        <v>1.0413926851582251</v>
-      </c>
-    </row>
-    <row r="12" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A12">
-        <v>12</v>
-      </c>
-      <c r="B12">
-        <v>6815</v>
-      </c>
-      <c r="C12">
-        <v>170594</v>
-      </c>
-      <c r="D12">
-        <v>262002</v>
-      </c>
-      <c r="E12">
-        <v>162</v>
-      </c>
-      <c r="F12">
-        <v>324</v>
-      </c>
-      <c r="G12">
-        <v>101</v>
-      </c>
-      <c r="H12">
-        <v>81</v>
-      </c>
-      <c r="I12">
-        <v>154</v>
-      </c>
-      <c r="J12">
-        <v>12</v>
-      </c>
-      <c r="M12">
-        <f t="shared" si="3"/>
-        <v>3.8334658601706924</v>
-      </c>
-      <c r="N12">
-        <f t="shared" si="0"/>
-        <v>5.2319637524310654</v>
-      </c>
-      <c r="O12">
-        <f t="shared" si="0"/>
-        <v>5.4183046065321445</v>
-      </c>
-      <c r="R12">
-        <f t="shared" si="4"/>
-        <v>2.2095150145426308</v>
-      </c>
-      <c r="S12">
-        <f t="shared" si="1"/>
-        <v>2.510545010206612</v>
-      </c>
-      <c r="T12">
-        <f t="shared" si="1"/>
-        <v>2.0043213737826426</v>
-      </c>
-      <c r="W12">
-        <f t="shared" si="5"/>
-        <v>1.9084850188786497</v>
-      </c>
-      <c r="X12">
-        <f t="shared" si="2"/>
-        <v>2.1875207208364631</v>
-      </c>
-      <c r="Y12">
-        <f t="shared" si="2"/>
-        <v>1.0791812460476249</v>
-      </c>
-    </row>
-    <row r="13" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A13">
-        <v>13</v>
-      </c>
-      <c r="B13">
-        <v>9194</v>
-      </c>
-      <c r="C13">
-        <v>245435</v>
-      </c>
-      <c r="D13">
-        <v>380653</v>
-      </c>
-      <c r="E13">
-        <v>176</v>
-      </c>
-      <c r="F13">
-        <v>358</v>
-      </c>
-      <c r="G13">
-        <v>116</v>
-      </c>
-      <c r="H13">
-        <v>88</v>
-      </c>
-      <c r="I13">
-        <v>167</v>
-      </c>
-      <c r="J13">
-        <v>13</v>
-      </c>
-      <c r="M13">
-        <f t="shared" si="3"/>
-        <v>3.9635044994142907</v>
-      </c>
-      <c r="N13">
-        <f t="shared" si="0"/>
-        <v>5.389936494915041</v>
-      </c>
-      <c r="O13">
-        <f t="shared" si="0"/>
-        <v>5.5805292569017242</v>
-      </c>
-      <c r="R13">
-        <f t="shared" si="4"/>
-        <v>2.2455126678141499</v>
-      </c>
-      <c r="S13">
-        <f t="shared" si="1"/>
-        <v>2.5538830266438746</v>
-      </c>
-      <c r="T13">
-        <f t="shared" si="1"/>
-        <v>2.0644579892269186</v>
-      </c>
-      <c r="W13">
-        <f t="shared" si="5"/>
-        <v>1.9444826721501687</v>
-      </c>
-      <c r="X13">
-        <f t="shared" si="2"/>
-        <v>2.2227164711475833</v>
-      </c>
-      <c r="Y13">
-        <f t="shared" si="2"/>
-        <v>1.1139433523068367</v>
-      </c>
-    </row>
-    <row r="14" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A14">
-        <v>14</v>
-      </c>
-      <c r="B14">
-        <v>12148</v>
-      </c>
-      <c r="C14">
-        <v>344387</v>
-      </c>
-      <c r="D14">
-        <v>538839</v>
-      </c>
-      <c r="E14">
-        <v>190</v>
-      </c>
-      <c r="F14">
-        <v>393</v>
-      </c>
-      <c r="G14">
-        <v>132</v>
-      </c>
-      <c r="H14">
-        <v>95</v>
-      </c>
-      <c r="I14">
-        <v>180</v>
-      </c>
-      <c r="J14">
-        <v>14</v>
-      </c>
-      <c r="M14">
-        <f t="shared" si="3"/>
-        <v>4.0845047832462278</v>
-      </c>
-      <c r="N14">
-        <f t="shared" si="0"/>
-        <v>5.5370467492426405</v>
-      </c>
-      <c r="O14">
-        <f t="shared" si="0"/>
-        <v>5.7314590214827037</v>
-      </c>
-      <c r="R14">
-        <f t="shared" si="4"/>
-        <v>2.2787536009528289</v>
-      </c>
-      <c r="S14">
-        <f t="shared" si="1"/>
-        <v>2.5943925503754266</v>
-      </c>
-      <c r="T14">
-        <f t="shared" si="1"/>
-        <v>2.12057393120585</v>
-      </c>
-      <c r="W14">
-        <f t="shared" si="5"/>
-        <v>1.9777236052888478</v>
-      </c>
-      <c r="X14">
-        <f t="shared" si="2"/>
-        <v>2.255272505103306</v>
-      </c>
-      <c r="Y14">
-        <f t="shared" si="2"/>
-        <v>1.146128035678238</v>
-      </c>
-    </row>
-    <row r="15" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A15">
-        <v>15</v>
-      </c>
-      <c r="B15">
-        <v>15763</v>
-      </c>
-      <c r="C15">
-        <v>472832</v>
-      </c>
-      <c r="D15">
-        <v>745704</v>
-      </c>
-      <c r="E15">
-        <v>204</v>
-      </c>
-      <c r="F15">
-        <v>429</v>
-      </c>
-      <c r="G15">
-        <v>149</v>
-      </c>
-      <c r="H15">
-        <v>102</v>
-      </c>
-      <c r="I15">
-        <v>193</v>
-      </c>
-      <c r="J15">
-        <v>15</v>
-      </c>
-      <c r="M15">
-        <f t="shared" si="3"/>
-        <v>4.1976388755555698</v>
-      </c>
-      <c r="N15">
-        <f t="shared" si="0"/>
-        <v>5.6747068607520914</v>
-      </c>
-      <c r="O15">
-        <f t="shared" si="0"/>
-        <v>5.8725664726779767</v>
-      </c>
-      <c r="R15">
-        <f t="shared" si="4"/>
-        <v>2.3096301674258988</v>
-      </c>
-      <c r="S15">
-        <f t="shared" si="1"/>
-        <v>2.6324572921847245</v>
-      </c>
-      <c r="T15">
-        <f t="shared" si="1"/>
-        <v>2.173186268412274</v>
-      </c>
-      <c r="W15">
-        <f t="shared" si="5"/>
-        <v>2.0086001717619175</v>
-      </c>
-      <c r="X15">
-        <f t="shared" si="2"/>
-        <v>2.2855573090077739</v>
-      </c>
-      <c r="Y15">
-        <f t="shared" si="2"/>
-        <v>1.1760912590556813</v>
-      </c>
-    </row>
-    <row r="16" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A16">
-        <v>16</v>
-      </c>
-      <c r="B16">
-        <v>20131</v>
-      </c>
-      <c r="C16">
-        <v>636896</v>
-      </c>
-      <c r="D16">
-        <v>1011704</v>
-      </c>
-      <c r="E16">
-        <v>218</v>
-      </c>
-      <c r="F16">
-        <v>466</v>
-      </c>
-      <c r="G16">
-        <v>167</v>
-      </c>
-      <c r="H16">
-        <v>109</v>
-      </c>
-      <c r="I16">
-        <v>206</v>
-      </c>
-      <c r="J16">
-        <v>16</v>
-      </c>
-      <c r="M16">
-        <f t="shared" si="3"/>
-        <v>4.3038653488427041</v>
-      </c>
-      <c r="N16">
-        <f t="shared" si="0"/>
-        <v>5.8040685213250036</v>
-      </c>
-      <c r="O16">
-        <f t="shared" si="0"/>
-        <v>6.0050534670785991</v>
-      </c>
-      <c r="R16">
-        <f t="shared" si="4"/>
-        <v>2.3384564936046046</v>
-      </c>
-      <c r="S16">
-        <f t="shared" si="1"/>
-        <v>2.6683859166900001</v>
-      </c>
-      <c r="T16">
-        <f t="shared" si="1"/>
-        <v>2.2227164711475833</v>
-      </c>
-      <c r="W16">
-        <f t="shared" si="5"/>
-        <v>2.0374264979406238</v>
-      </c>
-      <c r="X16">
-        <f t="shared" si="2"/>
-        <v>2.3138672203691533</v>
-      </c>
-      <c r="Y16">
-        <f t="shared" si="2"/>
-        <v>1.2041199826559248</v>
-      </c>
-    </row>
-    <row r="17" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A17">
-        <v>17</v>
-      </c>
-      <c r="B17">
-        <v>25350</v>
-      </c>
-      <c r="C17">
-        <v>843497</v>
-      </c>
-      <c r="D17">
-        <v>1348695</v>
-      </c>
-      <c r="E17">
-        <v>232</v>
-      </c>
-      <c r="F17">
-        <v>504</v>
-      </c>
-      <c r="G17">
-        <v>186</v>
-      </c>
-      <c r="H17">
-        <v>116</v>
-      </c>
-      <c r="I17">
-        <v>219</v>
-      </c>
-      <c r="J17">
-        <v>17</v>
-      </c>
-      <c r="M17">
-        <f t="shared" si="3"/>
-        <v>4.4039779636693543</v>
-      </c>
-      <c r="N17">
-        <f t="shared" si="0"/>
-        <v>5.926083542306575</v>
-      </c>
-      <c r="O17">
-        <f t="shared" si="0"/>
-        <v>6.1299137474529397</v>
-      </c>
-      <c r="R17">
-        <f t="shared" si="4"/>
-        <v>2.3654879848908998</v>
-      </c>
-      <c r="S17">
-        <f t="shared" si="1"/>
-        <v>2.7024305364455254</v>
-      </c>
-      <c r="T17">
-        <f t="shared" si="1"/>
-        <v>2.2695129442179165</v>
-      </c>
-      <c r="W17">
-        <f t="shared" si="5"/>
-        <v>2.0644579892269186</v>
-      </c>
-      <c r="X17">
-        <f t="shared" si="2"/>
-        <v>2.3404441148401185</v>
-      </c>
-      <c r="Y17">
-        <f t="shared" si="2"/>
-        <v>1.2304489213782739</v>
-      </c>
-    </row>
-    <row r="18" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A18">
-        <v>18</v>
-      </c>
-      <c r="B18">
-        <v>31524</v>
-      </c>
-      <c r="C18">
-        <v>1100393</v>
-      </c>
-      <c r="D18">
-        <v>1770021</v>
-      </c>
-      <c r="E18">
-        <v>246</v>
-      </c>
-      <c r="F18">
-        <v>543</v>
-      </c>
-      <c r="G18">
-        <v>206</v>
-      </c>
-      <c r="H18">
-        <v>123</v>
-      </c>
-      <c r="I18">
-        <v>232</v>
-      </c>
-      <c r="J18">
-        <v>18</v>
-      </c>
-      <c r="M18">
-        <f t="shared" si="3"/>
-        <v>4.4986413188336947</v>
-      </c>
-      <c r="N18">
-        <f t="shared" ref="N18:N20" si="6">LOG(C18)</f>
-        <v>6.0415478190213152</v>
-      </c>
-      <c r="O18">
-        <f t="shared" ref="O18:O20" si="7">LOG(D18)</f>
-        <v>6.2479784189776355</v>
-      </c>
-      <c r="R18">
-        <f t="shared" si="4"/>
-        <v>2.3909351071033793</v>
-      </c>
-      <c r="S18">
-        <f t="shared" ref="S18:S20" si="8">LOG(F18)</f>
-        <v>2.7347998295888472</v>
-      </c>
-      <c r="T18">
-        <f t="shared" ref="T18:T20" si="9">LOG(G18)</f>
-        <v>2.3138672203691533</v>
-      </c>
-      <c r="W18">
-        <f t="shared" si="5"/>
-        <v>2.0899051114393981</v>
-      </c>
-      <c r="X18">
-        <f t="shared" ref="X18:X20" si="10">LOG(I18)</f>
-        <v>2.3654879848908998</v>
-      </c>
-      <c r="Y18">
-        <f t="shared" ref="Y18:Y20" si="11">LOG(J18)</f>
-        <v>1.255272505103306</v>
-      </c>
-    </row>
-    <row r="19" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A19">
-        <v>19</v>
-      </c>
-      <c r="B19">
-        <v>38763</v>
-      </c>
-      <c r="C19">
-        <v>1416230</v>
-      </c>
-      <c r="D19">
-        <v>2290602</v>
-      </c>
-      <c r="E19">
-        <v>260</v>
-      </c>
-      <c r="F19">
-        <v>583</v>
-      </c>
-      <c r="G19">
-        <v>227</v>
-      </c>
-      <c r="H19">
-        <v>130</v>
-      </c>
-      <c r="I19">
-        <v>245</v>
-      </c>
-      <c r="J19">
-        <v>19</v>
-      </c>
-      <c r="M19">
-        <f t="shared" si="3"/>
-        <v>4.5884173812019249</v>
-      </c>
-      <c r="N19">
-        <f t="shared" si="6"/>
-        <v>6.151133789808104</v>
-      </c>
-      <c r="O19">
-        <f t="shared" si="7"/>
-        <v>6.3599496355798379</v>
-      </c>
-      <c r="R19">
-        <f t="shared" si="4"/>
-        <v>2.4149733479708178</v>
-      </c>
-      <c r="S19">
-        <f t="shared" si="8"/>
-        <v>2.7656685547590141</v>
-      </c>
-      <c r="T19">
-        <f t="shared" si="9"/>
-        <v>2.3560258571931225</v>
-      </c>
-      <c r="W19">
-        <f t="shared" si="5"/>
-        <v>2.1139433523068369</v>
-      </c>
-      <c r="X19">
-        <f t="shared" si="10"/>
-        <v>2.3891660843645326</v>
-      </c>
-      <c r="Y19">
-        <f t="shared" si="11"/>
-        <v>1.2787536009528289</v>
-      </c>
-    </row>
-    <row r="20" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A20">
-        <v>20</v>
-      </c>
-      <c r="B20">
-        <v>47183</v>
-      </c>
-      <c r="C20">
-        <v>1800590</v>
-      </c>
-      <c r="D20">
-        <v>2927022</v>
-      </c>
-      <c r="E20">
-        <v>274</v>
-      </c>
-      <c r="F20">
-        <v>624</v>
-      </c>
-      <c r="G20">
-        <v>249</v>
-      </c>
-      <c r="H20">
-        <v>137</v>
-      </c>
-      <c r="I20">
-        <v>258</v>
-      </c>
-      <c r="J20">
-        <v>20</v>
-      </c>
-      <c r="M20">
-        <f t="shared" si="3"/>
-        <v>4.6737855508358148</v>
-      </c>
-      <c r="N20">
-        <f t="shared" si="6"/>
-        <v>6.2554148338586577</v>
-      </c>
-      <c r="O20">
-        <f t="shared" si="7"/>
-        <v>6.4664259866779652</v>
-      </c>
-      <c r="R20">
-        <f t="shared" si="4"/>
-        <v>2.4377505628203879</v>
-      </c>
-      <c r="S20">
-        <f t="shared" si="8"/>
-        <v>2.7951845896824241</v>
-      </c>
-      <c r="T20">
-        <f t="shared" si="9"/>
-        <v>2.3961993470957363</v>
-      </c>
-      <c r="W20">
-        <f t="shared" si="5"/>
-        <v>2.1367205671564067</v>
-      </c>
-      <c r="X20">
-        <f t="shared" si="10"/>
-        <v>2.4116197059632301</v>
-      </c>
-      <c r="Y20">
-        <f t="shared" si="11"/>
-        <v>1.3010299956639813</v>
-      </c>
+    <row r="21" spans="1:49" x14ac:dyDescent="0.25">
+      <c r="E21" s="2"/>
+      <c r="F21" s="2"/>
+      <c r="G21" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
edited the comp.py to show only one subplot at a time
</commit_message>
<xml_diff>
--- a/ra/dataCounters/counters.xlsx
+++ b/ra/dataCounters/counters.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="A:\uni\masters nu\RA\pythonCode\ra\dataCounters\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE2EFA1B-18CF-4EC1-81A8-E4C86F644E5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C05E704F-4164-4413-B847-036682DABD4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -224,6 +224,11 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FF00FFFF"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -867,14 +872,26 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:rPr lang="en-US" b="1"/>
+              <a:rPr lang="en-US" sz="1600" b="1">
+                <a:solidFill>
+                  <a:schemeClr val="tx1"/>
+                </a:solidFill>
+              </a:rPr>
               <a:t>Log Count of</a:t>
             </a:r>
             <a:r>
-              <a:rPr lang="en-US" b="1" baseline="0"/>
+              <a:rPr lang="en-US" sz="1600" b="1" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1"/>
+                </a:solidFill>
+              </a:rPr>
               <a:t> Rotation Matrices vs N</a:t>
             </a:r>
-            <a:endParaRPr lang="en-US" b="1"/>
+            <a:endParaRPr lang="en-US" sz="1600" b="1">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+            </a:endParaRPr>
           </a:p>
         </c:rich>
       </c:tx>
@@ -1244,7 +1261,7 @@
           <c:spPr>
             <a:ln w="41275" cap="rnd">
               <a:solidFill>
-                <a:schemeClr val="accent3"/>
+                <a:schemeClr val="accent6"/>
               </a:solidFill>
               <a:round/>
             </a:ln>
@@ -1401,7 +1418,7 @@
           <c:spPr>
             <a:ln w="28575" cap="rnd">
               <a:solidFill>
-                <a:schemeClr val="accent4"/>
+                <a:srgbClr val="7030A0"/>
               </a:solidFill>
               <a:round/>
             </a:ln>
@@ -1492,7 +1509,7 @@
           <c:spPr>
             <a:ln w="28575" cap="rnd">
               <a:solidFill>
-                <a:schemeClr val="accent6"/>
+                <a:srgbClr val="00FFFF"/>
               </a:solidFill>
               <a:round/>
             </a:ln>
@@ -1593,6 +1610,20 @@
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
         <c:title>
           <c:tx>
             <c:rich>
@@ -1600,12 +1631,9 @@
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
-                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:defRPr sz="1600" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
-                      <a:schemeClr val="tx1">
-                        <a:lumMod val="65000"/>
-                        <a:lumOff val="35000"/>
-                      </a:schemeClr>
+                      <a:schemeClr val="tx1"/>
                     </a:solidFill>
                     <a:latin typeface="+mn-lt"/>
                     <a:ea typeface="+mn-ea"/>
@@ -1613,7 +1641,11 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:rPr lang="en-US" sz="1200" b="1"/>
+                  <a:rPr lang="en-US" sz="1600" b="1">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1"/>
+                    </a:solidFill>
+                  </a:rPr>
                   <a:t>N, Number of Links</a:t>
                 </a:r>
               </a:p>
@@ -1632,12 +1664,9 @@
             <a:lstStyle/>
             <a:p>
               <a:pPr>
-                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:defRPr sz="1600" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                   <a:solidFill>
-                    <a:schemeClr val="tx1">
-                      <a:lumMod val="65000"/>
-                      <a:lumOff val="35000"/>
-                    </a:schemeClr>
+                    <a:schemeClr val="tx1"/>
                   </a:solidFill>
                   <a:latin typeface="+mn-lt"/>
                   <a:ea typeface="+mn-ea"/>
@@ -1667,7 +1696,7 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="1200" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:defRPr sz="1400" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
                   <a:schemeClr val="tx1">
                     <a:lumMod val="65000"/>
@@ -1717,12 +1746,9 @@
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
-                  <a:defRPr sz="1200" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:defRPr sz="1600" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
-                      <a:schemeClr val="tx1">
-                        <a:lumMod val="65000"/>
-                        <a:lumOff val="35000"/>
-                      </a:schemeClr>
+                      <a:schemeClr val="tx1"/>
                     </a:solidFill>
                     <a:latin typeface="+mn-lt"/>
                     <a:ea typeface="+mn-ea"/>
@@ -1730,25 +1756,34 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:rPr lang="en-US" sz="1200" b="1"/>
+                  <a:rPr lang="en-US" sz="1600" b="1">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1"/>
+                    </a:solidFill>
+                  </a:rPr>
                   <a:t>Log</a:t>
                 </a:r>
                 <a:r>
-                  <a:rPr lang="en-US" sz="1200" b="1" baseline="0"/>
+                  <a:rPr lang="en-US" sz="1600" b="1" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1"/>
+                    </a:solidFill>
+                  </a:rPr>
                   <a:t> Count of </a:t>
                 </a:r>
                 <a:r>
-                  <a:rPr lang="en-US" sz="1200" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:rPr lang="en-US" sz="1600" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
-                      <a:sysClr val="windowText" lastClr="000000">
-                        <a:lumMod val="65000"/>
-                        <a:lumOff val="35000"/>
-                      </a:sysClr>
+                      <a:schemeClr val="tx1"/>
                     </a:solidFill>
                   </a:rPr>
                   <a:t>Rotation Matrices</a:t>
                 </a:r>
-                <a:endParaRPr lang="en-US" sz="1200" b="1"/>
+                <a:endParaRPr lang="en-US" sz="1600" b="1">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                </a:endParaRPr>
               </a:p>
             </c:rich>
           </c:tx>
@@ -1765,12 +1800,9 @@
             <a:lstStyle/>
             <a:p>
               <a:pPr>
-                <a:defRPr sz="1200" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:defRPr sz="1600" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                   <a:solidFill>
-                    <a:schemeClr val="tx1">
-                      <a:lumMod val="65000"/>
-                      <a:lumOff val="35000"/>
-                    </a:schemeClr>
+                    <a:schemeClr val="tx1"/>
                   </a:solidFill>
                   <a:latin typeface="+mn-lt"/>
                   <a:ea typeface="+mn-ea"/>
@@ -1799,7 +1831,7 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="1200" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:defRPr sz="1400" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
                   <a:schemeClr val="tx1">
                     <a:lumMod val="65000"/>
@@ -1991,7 +2023,17 @@
     </c:title>
     <c:autoTitleDeleted val="0"/>
     <c:plotArea>
-      <c:layout/>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="8.0327900188946963E-2"/>
+          <c:y val="0.14476423756943255"/>
+          <c:w val="0.90463319536038389"/>
+          <c:h val="0.71670393802656129"/>
+        </c:manualLayout>
+      </c:layout>
       <c:scatterChart>
         <c:scatterStyle val="lineMarker"/>
         <c:varyColors val="0"/>
@@ -2436,6 +2478,406 @@
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000002-2E4A-4135-80FD-2850A25A980E}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet1!$K$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>gibbs_AddCount</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="linear"/>
+            <c:dispRSqr val="0"/>
+            <c:dispEq val="1"/>
+            <c:trendlineLbl>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="-7.6735428069556128E-3"/>
+                  <c:y val="-8.2332711829293553E-2"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:numFmt formatCode="General" sourceLinked="0"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="65000"/>
+                          <a:lumOff val="35000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:latin typeface="+mn-lt"/>
+                      <a:ea typeface="+mn-ea"/>
+                      <a:cs typeface="+mn-cs"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="en-US"/>
+                </a:p>
+              </c:txPr>
+            </c:trendlineLbl>
+          </c:trendline>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Sheet1!$A$2:$A$20</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="19"/>
+                <c:pt idx="0">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>11</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>13</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>14</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>17</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>18</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>19</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>20</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Sheet1!$K$2:$K$20</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="19"/>
+                <c:pt idx="0">
+                  <c:v>30</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>45</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>60</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>75</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>90</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>105</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>120</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>135</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>150</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>165</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>180</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>195</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>210</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>225</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>240</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>255</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>270</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>285</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>300</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-4CBA-4E4F-B27A-F2B0E5FEA109}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="3"/>
+          <c:order val="3"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet1!$N$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>lie_AddCount</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent4"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent4"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Sheet1!$A$2:$A$20</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="19"/>
+                <c:pt idx="0">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>11</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>13</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>14</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>17</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>18</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>19</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>20</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Sheet1!$N$2:$N$20</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="19"/>
+                <c:pt idx="0">
+                  <c:v>13</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>27</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>34</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>41</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>48</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>55</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>62</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>69</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>76</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>83</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>90</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>97</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>104</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>111</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>118</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>125</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>132</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>139</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000003-4CBA-4E4F-B27A-F2B0E5FEA109}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2742,8 +3184,8 @@
           <c:yMode val="edge"/>
           <c:x val="0.11003196634319017"/>
           <c:y val="0.15783933841821754"/>
-          <c:w val="0.20231670193768153"/>
-          <c:h val="0.21052776343844135"/>
+          <c:w val="0.15936309366609391"/>
+          <c:h val="0.36842358601727238"/>
         </c:manualLayout>
       </c:layout>
       <c:overlay val="1"/>
@@ -3571,51 +4013,6 @@
               <a:effectLst/>
             </c:spPr>
           </c:marker>
-          <c:trendline>
-            <c:spPr>
-              <a:ln w="19050" cap="rnd">
-                <a:solidFill>
-                  <a:schemeClr val="accent2"/>
-                </a:solidFill>
-                <a:prstDash val="sysDot"/>
-              </a:ln>
-              <a:effectLst/>
-            </c:spPr>
-            <c:trendlineType val="poly"/>
-            <c:order val="2"/>
-            <c:dispRSqr val="0"/>
-            <c:dispEq val="1"/>
-            <c:trendlineLbl>
-              <c:numFmt formatCode="General" sourceLinked="0"/>
-              <c:spPr>
-                <a:noFill/>
-                <a:ln>
-                  <a:noFill/>
-                </a:ln>
-                <a:effectLst/>
-              </c:spPr>
-              <c:txPr>
-                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-                <a:lstStyle/>
-                <a:p>
-                  <a:pPr>
-                    <a:defRPr sz="1200" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                      <a:solidFill>
-                        <a:schemeClr val="tx1">
-                          <a:lumMod val="65000"/>
-                          <a:lumOff val="35000"/>
-                        </a:schemeClr>
-                      </a:solidFill>
-                      <a:latin typeface="+mn-lt"/>
-                      <a:ea typeface="+mn-ea"/>
-                      <a:cs typeface="+mn-cs"/>
-                    </a:defRPr>
-                  </a:pPr>
-                  <a:endParaRPr lang="en-US"/>
-                </a:p>
-              </c:txPr>
-            </c:trendlineLbl>
-          </c:trendline>
           <c:xVal>
             <c:numRef>
               <c:f>Sheet1!$A$2:$A$20</c:f>
@@ -3791,26 +4188,196 @@
               <a:effectLst/>
             </c:spPr>
           </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Sheet1!$A$2:$A$20</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="19"/>
+                <c:pt idx="0">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>11</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>13</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>14</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>17</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>18</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>19</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>20</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Sheet1!$I$2:$I$20</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="19"/>
+                <c:pt idx="0">
+                  <c:v>24</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>37</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>50</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>63</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>76</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>89</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>102</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>115</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>128</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>141</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>154</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>167</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>180</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>193</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>206</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>219</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>232</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>245</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>258</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000003-B2A3-467A-9206-586B1E479F89}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet1!$L$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>gibbs_MultCount</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
           <c:trendline>
             <c:spPr>
               <a:ln w="19050" cap="rnd">
                 <a:solidFill>
-                  <a:schemeClr val="accent3"/>
+                  <a:schemeClr val="accent1"/>
                 </a:solidFill>
                 <a:prstDash val="sysDot"/>
               </a:ln>
               <a:effectLst/>
             </c:spPr>
-            <c:trendlineType val="linear"/>
+            <c:trendlineType val="poly"/>
+            <c:order val="2"/>
             <c:dispRSqr val="0"/>
             <c:dispEq val="1"/>
             <c:trendlineLbl>
-              <c:layout>
-                <c:manualLayout>
-                  <c:x val="-3.6950296467178893E-2"/>
-                  <c:y val="9.7275547908637111E-4"/>
-                </c:manualLayout>
-              </c:layout>
               <c:numFmt formatCode="General" sourceLinked="0"/>
               <c:spPr>
                 <a:noFill/>
@@ -3824,7 +4391,7 @@
                 <a:lstStyle/>
                 <a:p>
                   <a:pPr>
-                    <a:defRPr sz="1200" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                       <a:solidFill>
                         <a:schemeClr val="tx1">
                           <a:lumMod val="65000"/>
@@ -3909,66 +4476,66 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Sheet1!$I$2:$I$20</c:f>
+              <c:f>Sheet1!$L$2:$L$20</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="19"/>
                 <c:pt idx="0">
-                  <c:v>24</c:v>
+                  <c:v>40</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>37</c:v>
+                  <c:v>60</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>50</c:v>
+                  <c:v>80</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>63</c:v>
+                  <c:v>100</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>76</c:v>
+                  <c:v>120</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>89</c:v>
+                  <c:v>140</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>102</c:v>
+                  <c:v>160</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>115</c:v>
+                  <c:v>180</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>128</c:v>
+                  <c:v>200</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>141</c:v>
+                  <c:v>220</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>154</c:v>
+                  <c:v>240</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>167</c:v>
+                  <c:v>260</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>180</c:v>
+                  <c:v>280</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>193</c:v>
+                  <c:v>300</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>206</c:v>
+                  <c:v>320</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>219</c:v>
+                  <c:v>340</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>232</c:v>
+                  <c:v>360</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>245</c:v>
+                  <c:v>380</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>258</c:v>
+                  <c:v>400</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3976,7 +4543,226 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000003-B2A3-467A-9206-586B1E479F89}"/>
+              <c16:uniqueId val="{00000002-5354-42EF-90A5-08EE8D7EA22E}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="3"/>
+          <c:order val="3"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet1!$O$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>lie_MultCount</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent4"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent4"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent4"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="linear"/>
+            <c:dispRSqr val="0"/>
+            <c:dispEq val="1"/>
+            <c:trendlineLbl>
+              <c:numFmt formatCode="General" sourceLinked="0"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="65000"/>
+                          <a:lumOff val="35000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:latin typeface="+mn-lt"/>
+                      <a:ea typeface="+mn-ea"/>
+                      <a:cs typeface="+mn-cs"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="en-US"/>
+                </a:p>
+              </c:txPr>
+            </c:trendlineLbl>
+          </c:trendline>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Sheet1!$A$2:$A$20</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="19"/>
+                <c:pt idx="0">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>11</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>13</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>14</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>17</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>18</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>19</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>20</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Sheet1!$O$2:$O$20</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="19"/>
+                <c:pt idx="0">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>38</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>51</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>64</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>77</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>90</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>103</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>116</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>129</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>142</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>155</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>168</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>181</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>194</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>207</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>220</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>233</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>246</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>259</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000003-5354-42EF-90A5-08EE8D7EA22E}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -4255,8 +5041,8 @@
           <c:yMode val="edge"/>
           <c:x val="0.11411552369513132"/>
           <c:y val="0.15783933841821757"/>
-          <c:w val="0.19984734958977585"/>
-          <c:h val="0.21052776343844135"/>
+          <c:w val="0.14884655619588774"/>
+          <c:h val="0.315791645157662"/>
         </c:manualLayout>
       </c:layout>
       <c:overlay val="1"/>
@@ -5049,57 +5835,6 @@
               <a:effectLst/>
             </c:spPr>
           </c:marker>
-          <c:trendline>
-            <c:spPr>
-              <a:ln w="19050" cap="rnd">
-                <a:solidFill>
-                  <a:schemeClr val="accent2"/>
-                </a:solidFill>
-                <a:prstDash val="sysDot"/>
-              </a:ln>
-              <a:effectLst/>
-            </c:spPr>
-            <c:trendlineType val="poly"/>
-            <c:order val="2"/>
-            <c:dispRSqr val="0"/>
-            <c:dispEq val="1"/>
-            <c:trendlineLbl>
-              <c:layout>
-                <c:manualLayout>
-                  <c:x val="-1.5910595921272554E-2"/>
-                  <c:y val="3.0969037347818192E-2"/>
-                </c:manualLayout>
-              </c:layout>
-              <c:numFmt formatCode="General" sourceLinked="0"/>
-              <c:spPr>
-                <a:noFill/>
-                <a:ln>
-                  <a:noFill/>
-                </a:ln>
-                <a:effectLst/>
-              </c:spPr>
-              <c:txPr>
-                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-                <a:lstStyle/>
-                <a:p>
-                  <a:pPr>
-                    <a:defRPr sz="1200" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                      <a:solidFill>
-                        <a:schemeClr val="tx1">
-                          <a:lumMod val="65000"/>
-                          <a:lumOff val="35000"/>
-                        </a:schemeClr>
-                      </a:solidFill>
-                      <a:latin typeface="+mn-lt"/>
-                      <a:ea typeface="+mn-ea"/>
-                      <a:cs typeface="+mn-cs"/>
-                    </a:defRPr>
-                  </a:pPr>
-                  <a:endParaRPr lang="en-US"/>
-                </a:p>
-              </c:txPr>
-            </c:trendlineLbl>
-          </c:trendline>
           <c:xVal>
             <c:numRef>
               <c:f>Sheet1!$A$2:$A$20</c:f>
@@ -5275,11 +6010,186 @@
               <a:effectLst/>
             </c:spPr>
           </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Sheet1!$A$2:$A$20</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="19"/>
+                <c:pt idx="0">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>11</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>13</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>14</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>17</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>18</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>19</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>20</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Sheet1!$J$2:$J$20</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="19"/>
+                <c:pt idx="0">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>11</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>13</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>14</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>17</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>18</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>19</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>20</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000003-FC98-4C51-91A9-5CF25CC53A49}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet1!$M$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>gibbs_TrigCount</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
           <c:trendline>
             <c:spPr>
               <a:ln w="19050" cap="rnd">
                 <a:solidFill>
-                  <a:schemeClr val="accent3"/>
+                  <a:schemeClr val="accent1"/>
                 </a:solidFill>
                 <a:prstDash val="sysDot"/>
               </a:ln>
@@ -5289,12 +6199,6 @@
             <c:dispRSqr val="0"/>
             <c:dispEq val="1"/>
             <c:trendlineLbl>
-              <c:layout>
-                <c:manualLayout>
-                  <c:x val="-4.8017260554295123E-2"/>
-                  <c:y val="-4.4743068288367847E-2"/>
-                </c:manualLayout>
-              </c:layout>
               <c:numFmt formatCode="General" sourceLinked="0"/>
               <c:spPr>
                 <a:noFill/>
@@ -5308,7 +6212,7 @@
                 <a:lstStyle/>
                 <a:p>
                   <a:pPr>
-                    <a:defRPr sz="1200" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                       <a:solidFill>
                         <a:schemeClr val="tx1">
                           <a:lumMod val="65000"/>
@@ -5393,66 +6297,66 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Sheet1!$J$2:$J$20</c:f>
+              <c:f>Sheet1!$M$2:$M$20</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="19"/>
                 <c:pt idx="0">
-                  <c:v>2</c:v>
+                  <c:v>6</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>3</c:v>
+                  <c:v>9</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>4</c:v>
+                  <c:v>12</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5</c:v>
+                  <c:v>15</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>6</c:v>
+                  <c:v>18</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>7</c:v>
+                  <c:v>21</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>8</c:v>
+                  <c:v>24</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>9</c:v>
+                  <c:v>27</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>10</c:v>
+                  <c:v>30</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>11</c:v>
+                  <c:v>33</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>12</c:v>
+                  <c:v>36</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>13</c:v>
+                  <c:v>39</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>14</c:v>
+                  <c:v>42</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>15</c:v>
+                  <c:v>45</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>16</c:v>
+                  <c:v>48</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>17</c:v>
+                  <c:v>51</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>18</c:v>
+                  <c:v>54</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>19</c:v>
+                  <c:v>57</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>20</c:v>
+                  <c:v>60</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -5460,7 +6364,226 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000003-FC98-4C51-91A9-5CF25CC53A49}"/>
+              <c16:uniqueId val="{00000002-13FD-4BDB-8291-2605049DB2F0}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="3"/>
+          <c:order val="3"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet1!$P$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>lie_TrigCount</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent4"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent4"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent4"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="linear"/>
+            <c:dispRSqr val="0"/>
+            <c:dispEq val="1"/>
+            <c:trendlineLbl>
+              <c:numFmt formatCode="General" sourceLinked="0"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="65000"/>
+                          <a:lumOff val="35000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:latin typeface="+mn-lt"/>
+                      <a:ea typeface="+mn-ea"/>
+                      <a:cs typeface="+mn-cs"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="en-US"/>
+                </a:p>
+              </c:txPr>
+            </c:trendlineLbl>
+          </c:trendline>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Sheet1!$A$2:$A$20</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="19"/>
+                <c:pt idx="0">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>11</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>13</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>14</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>17</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>18</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>19</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>20</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Sheet1!$P$2:$P$20</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="19"/>
+                <c:pt idx="0">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>11</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>19</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>23</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>27</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>31</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>35</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>39</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>43</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>47</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>51</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>55</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>59</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>63</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>67</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>71</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>75</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>79</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000003-13FD-4BDB-8291-2605049DB2F0}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -5719,25 +6842,11 @@
     </c:plotArea>
     <c:legend>
       <c:legendPos val="r"/>
-      <c:layout>
-        <c:manualLayout>
-          <c:xMode val="edge"/>
-          <c:yMode val="edge"/>
-          <c:x val="0.1571825132027988"/>
-          <c:y val="0.23581203839547649"/>
-          <c:w val="0.19390707517492517"/>
-          <c:h val="0.21052776343844135"/>
-        </c:manualLayout>
-      </c:layout>
       <c:overlay val="1"/>
       <c:spPr>
-        <a:solidFill>
-          <a:schemeClr val="bg1"/>
-        </a:solidFill>
+        <a:noFill/>
         <a:ln>
-          <a:solidFill>
-            <a:schemeClr val="tx1"/>
-          </a:solidFill>
+          <a:noFill/>
         </a:ln>
         <a:effectLst/>
       </c:spPr>
@@ -5829,10 +6938,7 @@
             <a:pPr>
               <a:defRPr sz="1400" b="1" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
                 <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
-                  </a:schemeClr>
+                  <a:schemeClr val="tx1"/>
                 </a:solidFill>
                 <a:latin typeface="+mn-lt"/>
                 <a:ea typeface="+mn-ea"/>
@@ -5840,14 +6946,26 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:rPr lang="en-US" b="1"/>
+              <a:rPr lang="en-US" sz="1600" b="1">
+                <a:solidFill>
+                  <a:schemeClr val="tx1"/>
+                </a:solidFill>
+              </a:rPr>
               <a:t>Log Count of</a:t>
             </a:r>
             <a:r>
-              <a:rPr lang="en-US" b="1" baseline="0"/>
+              <a:rPr lang="en-US" sz="1600" b="1" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1"/>
+                </a:solidFill>
+              </a:rPr>
               <a:t> Additions vs N</a:t>
             </a:r>
-            <a:endParaRPr lang="en-US" b="1"/>
+            <a:endParaRPr lang="en-US" sz="1600" b="1">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+            </a:endParaRPr>
           </a:p>
         </c:rich>
       </c:tx>
@@ -5866,10 +6984,7 @@
           <a:pPr>
             <a:defRPr sz="1400" b="1" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
               <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="65000"/>
-                  <a:lumOff val="35000"/>
-                </a:schemeClr>
+                <a:schemeClr val="tx1"/>
               </a:solidFill>
               <a:latin typeface="+mn-lt"/>
               <a:ea typeface="+mn-ea"/>
@@ -6209,7 +7324,7 @@
           <c:spPr>
             <a:ln w="41275" cap="rnd">
               <a:solidFill>
-                <a:schemeClr val="accent3"/>
+                <a:schemeClr val="accent6"/>
               </a:solidFill>
               <a:round/>
             </a:ln>
@@ -6366,7 +7481,7 @@
           <c:spPr>
             <a:ln w="28575" cap="rnd">
               <a:solidFill>
-                <a:schemeClr val="accent4"/>
+                <a:srgbClr val="7030A0"/>
               </a:solidFill>
               <a:round/>
             </a:ln>
@@ -6457,7 +7572,7 @@
           <c:spPr>
             <a:ln w="28575" cap="rnd">
               <a:solidFill>
-                <a:schemeClr val="accent6"/>
+                <a:srgbClr val="00FFFF"/>
               </a:solidFill>
               <a:round/>
             </a:ln>
@@ -6558,6 +7673,20 @@
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
         <c:title>
           <c:tx>
             <c:rich>
@@ -6567,10 +7696,7 @@
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
-                      <a:schemeClr val="tx1">
-                        <a:lumMod val="65000"/>
-                        <a:lumOff val="35000"/>
-                      </a:schemeClr>
+                      <a:schemeClr val="tx1"/>
                     </a:solidFill>
                     <a:latin typeface="+mn-lt"/>
                     <a:ea typeface="+mn-ea"/>
@@ -6578,7 +7704,11 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:rPr lang="en-US" sz="1200" b="1"/>
+                  <a:rPr lang="en-US" sz="1600" b="1">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1"/>
+                    </a:solidFill>
+                  </a:rPr>
                   <a:t>N, Number of Links</a:t>
                 </a:r>
               </a:p>
@@ -6599,10 +7729,7 @@
               <a:pPr>
                 <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                   <a:solidFill>
-                    <a:schemeClr val="tx1">
-                      <a:lumMod val="65000"/>
-                      <a:lumOff val="35000"/>
-                    </a:schemeClr>
+                    <a:schemeClr val="tx1"/>
                   </a:solidFill>
                   <a:latin typeface="+mn-lt"/>
                   <a:ea typeface="+mn-ea"/>
@@ -6632,7 +7759,7 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="1200" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:defRPr sz="1400" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
                   <a:schemeClr val="tx1">
                     <a:lumMod val="65000"/>
@@ -6684,10 +7811,7 @@
                 <a:pPr>
                   <a:defRPr sz="1200" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
-                      <a:schemeClr val="tx1">
-                        <a:lumMod val="65000"/>
-                        <a:lumOff val="35000"/>
-                      </a:schemeClr>
+                      <a:schemeClr val="tx1"/>
                     </a:solidFill>
                     <a:latin typeface="+mn-lt"/>
                     <a:ea typeface="+mn-ea"/>
@@ -6695,14 +7819,26 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:rPr lang="en-US" sz="1200" b="1"/>
+                  <a:rPr lang="en-US" sz="1600" b="1">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1"/>
+                    </a:solidFill>
+                  </a:rPr>
                   <a:t>Log</a:t>
                 </a:r>
                 <a:r>
-                  <a:rPr lang="en-US" sz="1200" b="1" baseline="0"/>
+                  <a:rPr lang="en-US" sz="1600" b="1" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1"/>
+                    </a:solidFill>
+                  </a:rPr>
                   <a:t> Count of Additions</a:t>
                 </a:r>
-                <a:endParaRPr lang="en-US" sz="1200" b="1"/>
+                <a:endParaRPr lang="en-US" sz="1600" b="1">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                </a:endParaRPr>
               </a:p>
             </c:rich>
           </c:tx>
@@ -6721,10 +7857,7 @@
               <a:pPr>
                 <a:defRPr sz="1200" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                   <a:solidFill>
-                    <a:schemeClr val="tx1">
-                      <a:lumMod val="65000"/>
-                      <a:lumOff val="35000"/>
-                    </a:schemeClr>
+                    <a:schemeClr val="tx1"/>
                   </a:solidFill>
                   <a:latin typeface="+mn-lt"/>
                   <a:ea typeface="+mn-ea"/>
@@ -6753,7 +7886,7 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="1200" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:defRPr sz="1400" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
                   <a:schemeClr val="tx1">
                     <a:lumMod val="65000"/>
@@ -6771,6 +7904,7 @@
         <c:crossAx val="1130468127"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
+        <c:majorUnit val="1"/>
       </c:valAx>
       <c:spPr>
         <a:noFill/>
@@ -6786,8 +7920,8 @@
         <c:manualLayout>
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
-          <c:x val="0.18056261061456588"/>
-          <c:y val="0.170133005526208"/>
+          <c:x val="0.11667336162403484"/>
+          <c:y val="0.12231303365560316"/>
           <c:w val="0.15688977522976036"/>
           <c:h val="0.23987374712489298"/>
         </c:manualLayout>
@@ -7772,14 +8906,26 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:rPr lang="en-US" b="1"/>
+              <a:rPr lang="en-US" sz="1600" b="1">
+                <a:solidFill>
+                  <a:schemeClr val="tx1"/>
+                </a:solidFill>
+              </a:rPr>
               <a:t>Log Count of</a:t>
             </a:r>
             <a:r>
-              <a:rPr lang="en-US" b="1" baseline="0"/>
+              <a:rPr lang="en-US" sz="1600" b="1" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1"/>
+                </a:solidFill>
+              </a:rPr>
               <a:t> Multiplications vs N</a:t>
             </a:r>
-            <a:endParaRPr lang="en-US" b="1"/>
+            <a:endParaRPr lang="en-US" sz="1600" b="1">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+            </a:endParaRPr>
           </a:p>
         </c:rich>
       </c:tx>
@@ -8141,7 +9287,7 @@
           <c:spPr>
             <a:ln w="41275" cap="rnd">
               <a:solidFill>
-                <a:schemeClr val="accent3"/>
+                <a:schemeClr val="accent6"/>
               </a:solidFill>
               <a:round/>
             </a:ln>
@@ -8298,7 +9444,7 @@
           <c:spPr>
             <a:ln w="28575" cap="rnd">
               <a:solidFill>
-                <a:schemeClr val="accent4"/>
+                <a:srgbClr val="7030A0"/>
               </a:solidFill>
               <a:round/>
             </a:ln>
@@ -8389,7 +9535,7 @@
           <c:spPr>
             <a:ln w="28575" cap="rnd">
               <a:solidFill>
-                <a:schemeClr val="accent6"/>
+                <a:srgbClr val="00FFFF"/>
               </a:solidFill>
               <a:round/>
             </a:ln>
@@ -8490,6 +9636,20 @@
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
         <c:title>
           <c:tx>
             <c:rich>
@@ -8497,12 +9657,9 @@
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
-                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:defRPr sz="1600" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
-                      <a:schemeClr val="tx1">
-                        <a:lumMod val="65000"/>
-                        <a:lumOff val="35000"/>
-                      </a:schemeClr>
+                      <a:schemeClr val="tx1"/>
                     </a:solidFill>
                     <a:latin typeface="+mn-lt"/>
                     <a:ea typeface="+mn-ea"/>
@@ -8510,7 +9667,11 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:rPr lang="en-US" sz="1200" b="1"/>
+                  <a:rPr lang="en-US" sz="1600" b="1">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1"/>
+                    </a:solidFill>
+                  </a:rPr>
                   <a:t>N, Number of Links</a:t>
                 </a:r>
               </a:p>
@@ -8529,12 +9690,9 @@
             <a:lstStyle/>
             <a:p>
               <a:pPr>
-                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:defRPr sz="1600" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                   <a:solidFill>
-                    <a:schemeClr val="tx1">
-                      <a:lumMod val="65000"/>
-                      <a:lumOff val="35000"/>
-                    </a:schemeClr>
+                    <a:schemeClr val="tx1"/>
                   </a:solidFill>
                   <a:latin typeface="+mn-lt"/>
                   <a:ea typeface="+mn-ea"/>
@@ -8564,7 +9722,7 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="1200" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:defRPr sz="1400" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
                   <a:schemeClr val="tx1">
                     <a:lumMod val="65000"/>
@@ -8614,12 +9772,9 @@
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
-                  <a:defRPr sz="1200" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:defRPr sz="1600" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
-                      <a:schemeClr val="tx1">
-                        <a:lumMod val="65000"/>
-                        <a:lumOff val="35000"/>
-                      </a:schemeClr>
+                      <a:schemeClr val="tx1"/>
                     </a:solidFill>
                     <a:latin typeface="+mn-lt"/>
                     <a:ea typeface="+mn-ea"/>
@@ -8627,14 +9782,26 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:rPr lang="en-US" sz="1200" b="1"/>
+                  <a:rPr lang="en-US" sz="1600" b="1">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1"/>
+                    </a:solidFill>
+                  </a:rPr>
                   <a:t>Log</a:t>
                 </a:r>
                 <a:r>
-                  <a:rPr lang="en-US" sz="1200" b="1" baseline="0"/>
+                  <a:rPr lang="en-US" sz="1600" b="1" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1"/>
+                    </a:solidFill>
+                  </a:rPr>
                   <a:t> Count of Multiplications</a:t>
                 </a:r>
-                <a:endParaRPr lang="en-US" sz="1200" b="1"/>
+                <a:endParaRPr lang="en-US" sz="1600" b="1">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                </a:endParaRPr>
               </a:p>
             </c:rich>
           </c:tx>
@@ -8651,12 +9818,9 @@
             <a:lstStyle/>
             <a:p>
               <a:pPr>
-                <a:defRPr sz="1200" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:defRPr sz="1600" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                   <a:solidFill>
-                    <a:schemeClr val="tx1">
-                      <a:lumMod val="65000"/>
-                      <a:lumOff val="35000"/>
-                    </a:schemeClr>
+                    <a:schemeClr val="tx1"/>
                   </a:solidFill>
                   <a:latin typeface="+mn-lt"/>
                   <a:ea typeface="+mn-ea"/>
@@ -8685,7 +9849,7 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="1200" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:defRPr sz="1400" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
                   <a:schemeClr val="tx1">
                     <a:lumMod val="65000"/>
@@ -14576,16 +15740,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>18</xdr:col>
-      <xdr:colOff>542924</xdr:colOff>
-      <xdr:row>21</xdr:row>
-      <xdr:rowOff>95250</xdr:rowOff>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>363008</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>21167</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>31</xdr:col>
-      <xdr:colOff>514349</xdr:colOff>
-      <xdr:row>45</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
+      <xdr:col>32</xdr:col>
+      <xdr:colOff>334432</xdr:colOff>
+      <xdr:row>46</xdr:row>
+      <xdr:rowOff>154517</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -14749,8 +15913,8 @@
       <sheetName val="90s 9000"/>
     </sheetNames>
     <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1"/>
+      <sheetData sheetId="0" refreshError="1"/>
+      <sheetData sheetId="1" refreshError="1"/>
       <sheetData sheetId="2">
         <row r="2">
           <cell r="A2">
@@ -14848,15 +16012,15 @@
           </cell>
         </row>
       </sheetData>
-      <sheetData sheetId="3"/>
-      <sheetData sheetId="4"/>
-      <sheetData sheetId="5"/>
-      <sheetData sheetId="6"/>
-      <sheetData sheetId="7"/>
-      <sheetData sheetId="8"/>
-      <sheetData sheetId="9"/>
-      <sheetData sheetId="10"/>
-      <sheetData sheetId="11"/>
+      <sheetData sheetId="3" refreshError="1"/>
+      <sheetData sheetId="4" refreshError="1"/>
+      <sheetData sheetId="5" refreshError="1"/>
+      <sheetData sheetId="6" refreshError="1"/>
+      <sheetData sheetId="7" refreshError="1"/>
+      <sheetData sheetId="8" refreshError="1"/>
+      <sheetData sheetId="9" refreshError="1"/>
+      <sheetData sheetId="10" refreshError="1"/>
+      <sheetData sheetId="11" refreshError="1"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -15306,39 +16470,39 @@
         <v>7</v>
       </c>
       <c r="AA2">
-        <f>LOG(B2)</f>
+        <f t="shared" ref="AA2:AA20" si="0">LOG(B2)</f>
         <v>1.3010299956639813</v>
       </c>
       <c r="AB2">
-        <f>LOG(C2)</f>
+        <f t="shared" ref="AB2:AB20" si="1">LOG(C2)</f>
         <v>2.0530784434834195</v>
       </c>
       <c r="AC2">
-        <f>LOG(D2)</f>
+        <f t="shared" ref="AC2:AC20" si="2">LOG(D2)</f>
         <v>2.1492191126553797</v>
       </c>
       <c r="AF2">
-        <f>LOG(E2)</f>
+        <f t="shared" ref="AF2:AF20" si="3">LOG(E2)</f>
         <v>1.3424226808222062</v>
       </c>
       <c r="AG2">
-        <f>LOG(F2)</f>
+        <f t="shared" ref="AG2:AG20" si="4">LOG(F2)</f>
         <v>1.5910646070264991</v>
       </c>
       <c r="AH2">
-        <f>LOG(G2)</f>
+        <f t="shared" ref="AH2:AH20" si="5">LOG(G2)</f>
         <v>0.77815125038364363</v>
       </c>
       <c r="AK2">
-        <f>LOG(H2)</f>
+        <f t="shared" ref="AK2:AK20" si="6">LOG(H2)</f>
         <v>1.0413926851582251</v>
       </c>
       <c r="AL2">
-        <f>LOG(I2)</f>
+        <f t="shared" ref="AL2:AL20" si="7">LOG(I2)</f>
         <v>1.3802112417116059</v>
       </c>
       <c r="AM2">
-        <f>LOG(J2)</f>
+        <f t="shared" ref="AM2:AM20" si="8">LOG(J2)</f>
         <v>0.3010299956639812</v>
       </c>
       <c r="AP2">
@@ -15346,11 +16510,11 @@
         <v>1.4771212547196624</v>
       </c>
       <c r="AQ2">
-        <f t="shared" ref="AQ2:AR17" si="0">LOG(L2)</f>
+        <f t="shared" ref="AQ2:AR17" si="9">LOG(L2)</f>
         <v>1.6020599913279623</v>
       </c>
       <c r="AR2">
-        <f t="shared" si="0"/>
+        <f t="shared" si="9"/>
         <v>0.77815125038364363</v>
       </c>
       <c r="AU2">
@@ -15358,11 +16522,11 @@
         <v>1.1139433523068367</v>
       </c>
       <c r="AV2">
-        <f t="shared" ref="AV2:AW17" si="1">LOG(O2)</f>
+        <f t="shared" ref="AV2:AW17" si="10">LOG(O2)</f>
         <v>1.3979400086720377</v>
       </c>
       <c r="AW2">
-        <f t="shared" si="1"/>
+        <f t="shared" si="10"/>
         <v>0.84509804001425681</v>
       </c>
     </row>
@@ -15416,63 +16580,63 @@
         <v>11</v>
       </c>
       <c r="AA3">
-        <f>LOG(B3)</f>
+        <f t="shared" si="0"/>
         <v>1.7708520116421442</v>
       </c>
       <c r="AB3">
-        <f>LOG(C3)</f>
+        <f t="shared" si="1"/>
         <v>2.6937269489236471</v>
       </c>
       <c r="AC3">
-        <f>LOG(D3)</f>
+        <f t="shared" si="2"/>
         <v>2.8075350280688531</v>
       </c>
       <c r="AF3">
-        <f>LOG(E3)</f>
+        <f t="shared" si="3"/>
         <v>1.5563025007672873</v>
       </c>
       <c r="AG3">
-        <f>LOG(F3)</f>
+        <f t="shared" si="4"/>
         <v>1.7993405494535817</v>
       </c>
       <c r="AH3">
-        <f>LOG(G3)</f>
+        <f t="shared" si="5"/>
         <v>1.0413926851582251</v>
       </c>
       <c r="AK3">
-        <f>LOG(H3)</f>
+        <f t="shared" si="6"/>
         <v>1.255272505103306</v>
       </c>
       <c r="AL3">
-        <f>LOG(I3)</f>
+        <f t="shared" si="7"/>
         <v>1.568201724066995</v>
       </c>
       <c r="AM3">
-        <f>LOG(J3)</f>
+        <f t="shared" si="8"/>
         <v>0.47712125471966244</v>
       </c>
       <c r="AP3">
-        <f t="shared" ref="AP3:AP20" si="2">LOG(K3)</f>
+        <f t="shared" ref="AP3:AP20" si="11">LOG(K3)</f>
         <v>1.6532125137753437</v>
       </c>
       <c r="AQ3">
-        <f t="shared" si="0"/>
+        <f t="shared" si="9"/>
         <v>1.7781512503836436</v>
       </c>
       <c r="AR3">
-        <f t="shared" si="0"/>
+        <f t="shared" si="9"/>
         <v>0.95424250943932487</v>
       </c>
       <c r="AU3">
-        <f t="shared" ref="AU3:AU20" si="3">LOG(N3)</f>
+        <f t="shared" ref="AU3:AU20" si="12">LOG(N3)</f>
         <v>1.3010299956639813</v>
       </c>
       <c r="AV3">
-        <f t="shared" si="1"/>
+        <f t="shared" si="10"/>
         <v>1.5797835966168101</v>
       </c>
       <c r="AW3">
-        <f t="shared" si="1"/>
+        <f t="shared" si="10"/>
         <v>1.0413926851582251</v>
       </c>
     </row>
@@ -15526,63 +16690,63 @@
         <v>15</v>
       </c>
       <c r="AA4">
-        <f>LOG(B4)</f>
+        <f t="shared" si="0"/>
         <v>2.1553360374650619</v>
       </c>
       <c r="AB4">
-        <f>LOG(C4)</f>
+        <f t="shared" si="1"/>
         <v>3.1835545336188615</v>
       </c>
       <c r="AC4">
-        <f>LOG(D4)</f>
+        <f t="shared" si="2"/>
         <v>3.3092041796704077</v>
       </c>
       <c r="AF4">
-        <f>LOG(E4)</f>
+        <f t="shared" si="3"/>
         <v>1.6989700043360187</v>
       </c>
       <c r="AG4">
-        <f>LOG(F4)</f>
+        <f t="shared" si="4"/>
         <v>1.9444826721501687</v>
       </c>
       <c r="AH4">
-        <f>LOG(G4)</f>
+        <f t="shared" si="5"/>
         <v>1.2304489213782739</v>
       </c>
       <c r="AK4">
-        <f>LOG(H4)</f>
+        <f t="shared" si="6"/>
         <v>1.3979400086720377</v>
       </c>
       <c r="AL4">
-        <f>LOG(I4)</f>
+        <f t="shared" si="7"/>
         <v>1.6989700043360187</v>
       </c>
       <c r="AM4">
-        <f>LOG(J4)</f>
+        <f t="shared" si="8"/>
         <v>0.6020599913279624</v>
       </c>
       <c r="AP4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="11"/>
         <v>1.7781512503836436</v>
       </c>
       <c r="AQ4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="9"/>
         <v>1.9030899869919435</v>
       </c>
       <c r="AR4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="9"/>
         <v>1.0791812460476249</v>
       </c>
       <c r="AU4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="12"/>
         <v>1.4313637641589874</v>
       </c>
       <c r="AV4">
-        <f t="shared" si="1"/>
+        <f t="shared" si="10"/>
         <v>1.7075701760979363</v>
       </c>
       <c r="AW4">
-        <f t="shared" si="1"/>
+        <f t="shared" si="10"/>
         <v>1.1760912590556813</v>
       </c>
     </row>
@@ -15636,63 +16800,63 @@
         <v>19</v>
       </c>
       <c r="AA5">
-        <f>LOG(B5)</f>
+        <f t="shared" si="0"/>
         <v>2.4742162640762553</v>
       </c>
       <c r="AB5">
-        <f>LOG(C5)</f>
+        <f t="shared" si="1"/>
         <v>3.5787537844264348</v>
       </c>
       <c r="AC5">
-        <f>LOG(D5)</f>
+        <f t="shared" si="2"/>
         <v>3.7154183225950561</v>
       </c>
       <c r="AF5">
-        <f>LOG(E5)</f>
+        <f t="shared" si="3"/>
         <v>1.8061799739838871</v>
       </c>
       <c r="AG5">
-        <f>LOG(F5)</f>
+        <f t="shared" si="4"/>
         <v>2.0569048513364727</v>
       </c>
       <c r="AH5">
-        <f>LOG(G5)</f>
+        <f t="shared" si="5"/>
         <v>1.3802112417116059</v>
       </c>
       <c r="AK5">
-        <f>LOG(H5)</f>
+        <f t="shared" si="6"/>
         <v>1.505149978319906</v>
       </c>
       <c r="AL5">
-        <f>LOG(I5)</f>
+        <f t="shared" si="7"/>
         <v>1.7993405494535817</v>
       </c>
       <c r="AM5">
-        <f>LOG(J5)</f>
+        <f t="shared" si="8"/>
         <v>0.69897000433601886</v>
       </c>
       <c r="AP5">
-        <f t="shared" si="2"/>
+        <f t="shared" si="11"/>
         <v>1.8750612633917001</v>
       </c>
       <c r="AQ5">
-        <f t="shared" si="0"/>
+        <f t="shared" si="9"/>
         <v>2</v>
       </c>
       <c r="AR5">
-        <f t="shared" si="0"/>
+        <f t="shared" si="9"/>
         <v>1.1760912590556813</v>
       </c>
       <c r="AU5">
-        <f t="shared" si="3"/>
+        <f t="shared" si="12"/>
         <v>1.5314789170422551</v>
       </c>
       <c r="AV5">
-        <f t="shared" si="1"/>
+        <f t="shared" si="10"/>
         <v>1.8061799739838871</v>
       </c>
       <c r="AW5">
-        <f t="shared" si="1"/>
+        <f t="shared" si="10"/>
         <v>1.2787536009528289</v>
       </c>
     </row>
@@ -15746,63 +16910,63 @@
         <v>23</v>
       </c>
       <c r="AA6">
-        <f>LOG(B6)</f>
+        <f t="shared" si="0"/>
         <v>2.7450747915820575</v>
       </c>
       <c r="AB6">
-        <f>LOG(C6)</f>
+        <f t="shared" si="1"/>
         <v>3.9103575572728775</v>
       </c>
       <c r="AC6">
-        <f>LOG(D6)</f>
+        <f t="shared" si="2"/>
         <v>4.0570191243227658</v>
       </c>
       <c r="AF6">
-        <f>LOG(E6)</f>
+        <f t="shared" si="3"/>
         <v>1.8920946026904804</v>
       </c>
       <c r="AG6">
-        <f>LOG(F6)</f>
+        <f t="shared" si="4"/>
         <v>2.1492191126553797</v>
       </c>
       <c r="AH6">
-        <f>LOG(G6)</f>
+        <f t="shared" si="5"/>
         <v>1.505149978319906</v>
       </c>
       <c r="AK6">
-        <f>LOG(H6)</f>
+        <f t="shared" si="6"/>
         <v>1.5910646070264991</v>
       </c>
       <c r="AL6">
-        <f>LOG(I6)</f>
+        <f t="shared" si="7"/>
         <v>1.8808135922807914</v>
       </c>
       <c r="AM6">
-        <f>LOG(J6)</f>
+        <f t="shared" si="8"/>
         <v>0.77815125038364363</v>
       </c>
       <c r="AP6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="11"/>
         <v>1.954242509439325</v>
       </c>
       <c r="AQ6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="9"/>
         <v>2.0791812460476247</v>
       </c>
       <c r="AR6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="9"/>
         <v>1.255272505103306</v>
       </c>
       <c r="AU6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="12"/>
         <v>1.6127838567197355</v>
       </c>
       <c r="AV6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="10"/>
         <v>1.8864907251724818</v>
       </c>
       <c r="AW6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="10"/>
         <v>1.3617278360175928</v>
       </c>
     </row>
@@ -15856,63 +17020,63 @@
         <v>27</v>
       </c>
       <c r="AA7">
-        <f>LOG(B7)</f>
+        <f t="shared" si="0"/>
         <v>2.9800033715837464</v>
       </c>
       <c r="AB7">
-        <f>LOG(C7)</f>
+        <f t="shared" si="1"/>
         <v>4.1963420201397685</v>
       </c>
       <c r="AC7">
-        <f>LOG(D7)</f>
+        <f t="shared" si="2"/>
         <v>4.3518735766208998</v>
       </c>
       <c r="AF7">
-        <f>LOG(E7)</f>
+        <f t="shared" si="3"/>
         <v>1.9637878273455553</v>
       </c>
       <c r="AG7">
-        <f>LOG(F7)</f>
+        <f t="shared" si="4"/>
         <v>2.2278867046136734</v>
       </c>
       <c r="AH7">
-        <f>LOG(G7)</f>
+        <f t="shared" si="5"/>
         <v>1.6127838567197355</v>
       </c>
       <c r="AK7">
-        <f>LOG(H7)</f>
+        <f t="shared" si="6"/>
         <v>1.6627578316815741</v>
       </c>
       <c r="AL7">
-        <f>LOG(I7)</f>
+        <f t="shared" si="7"/>
         <v>1.9493900066449128</v>
       </c>
       <c r="AM7">
-        <f>LOG(J7)</f>
+        <f t="shared" si="8"/>
         <v>0.84509804001425681</v>
       </c>
       <c r="AP7">
-        <f t="shared" si="2"/>
+        <f t="shared" si="11"/>
         <v>2.0211892990699383</v>
       </c>
       <c r="AQ7">
-        <f t="shared" si="0"/>
+        <f t="shared" si="9"/>
         <v>2.1461280356782382</v>
       </c>
       <c r="AR7">
-        <f t="shared" si="0"/>
+        <f t="shared" si="9"/>
         <v>1.3222192947339193</v>
       </c>
       <c r="AU7">
-        <f t="shared" si="3"/>
+        <f t="shared" si="12"/>
         <v>1.6812412373755872</v>
       </c>
       <c r="AV7">
-        <f t="shared" si="1"/>
+        <f t="shared" si="10"/>
         <v>1.954242509439325</v>
       </c>
       <c r="AW7">
-        <f t="shared" si="1"/>
+        <f t="shared" si="10"/>
         <v>1.4313637641589874</v>
       </c>
     </row>
@@ -15966,63 +17130,63 @@
         <v>31</v>
       </c>
       <c r="AA8">
-        <f>LOG(B8)</f>
+        <f t="shared" si="0"/>
         <v>3.1872386198314788</v>
       </c>
       <c r="AB8">
-        <f>LOG(C8)</f>
+        <f t="shared" si="1"/>
         <v>4.4479638302267448</v>
       </c>
       <c r="AC8">
-        <f>LOG(D8)</f>
+        <f t="shared" si="2"/>
         <v>4.611298362296429</v>
       </c>
       <c r="AF8">
-        <f>LOG(E8)</f>
+        <f t="shared" si="3"/>
         <v>2.0253058652647704</v>
       </c>
       <c r="AG8">
-        <f>LOG(F8)</f>
+        <f t="shared" si="4"/>
         <v>2.2966651902615309</v>
       </c>
       <c r="AH8">
-        <f>LOG(G8)</f>
+        <f t="shared" si="5"/>
         <v>1.7075701760979363</v>
       </c>
       <c r="AK8">
-        <f>LOG(H8)</f>
+        <f t="shared" si="6"/>
         <v>1.7242758696007889</v>
       </c>
       <c r="AL8">
-        <f>LOG(I8)</f>
+        <f t="shared" si="7"/>
         <v>2.0086001717619175</v>
       </c>
       <c r="AM8">
-        <f>LOG(J8)</f>
+        <f t="shared" si="8"/>
         <v>0.90308998699194354</v>
       </c>
       <c r="AP8">
-        <f t="shared" si="2"/>
+        <f t="shared" si="11"/>
         <v>2.0791812460476247</v>
       </c>
       <c r="AQ8">
-        <f t="shared" si="0"/>
+        <f t="shared" si="9"/>
         <v>2.2041199826559246</v>
       </c>
       <c r="AR8">
-        <f t="shared" si="0"/>
+        <f t="shared" si="9"/>
         <v>1.3802112417116059</v>
       </c>
       <c r="AU8">
-        <f t="shared" si="3"/>
+        <f t="shared" si="12"/>
         <v>1.7403626894942439</v>
       </c>
       <c r="AV8">
-        <f t="shared" si="1"/>
+        <f t="shared" si="10"/>
         <v>2.012837224705172</v>
       </c>
       <c r="AW8">
-        <f t="shared" si="1"/>
+        <f t="shared" si="10"/>
         <v>1.4913616938342726</v>
       </c>
     </row>
@@ -16076,63 +17240,63 @@
         <v>35</v>
       </c>
       <c r="AA9">
-        <f>LOG(B9)</f>
+        <f t="shared" si="0"/>
         <v>3.3725438007590705</v>
       </c>
       <c r="AB9">
-        <f>LOG(C9)</f>
+        <f t="shared" si="1"/>
         <v>4.672734971642158</v>
       </c>
       <c r="AC9">
-        <f>LOG(D9)</f>
+        <f t="shared" si="2"/>
         <v>4.8429273560990236</v>
       </c>
       <c r="AF9">
-        <f>LOG(E9)</f>
+        <f t="shared" si="3"/>
         <v>2.0791812460476247</v>
       </c>
       <c r="AG9">
-        <f>LOG(F9)</f>
+        <f t="shared" si="4"/>
         <v>2.357934847000454</v>
       </c>
       <c r="AH9">
-        <f>LOG(G9)</f>
+        <f t="shared" si="5"/>
         <v>1.7923916894982539</v>
       </c>
       <c r="AK9">
-        <f>LOG(H9)</f>
+        <f t="shared" si="6"/>
         <v>1.7781512503836436</v>
       </c>
       <c r="AL9">
-        <f>LOG(I9)</f>
+        <f t="shared" si="7"/>
         <v>2.0606978403536118</v>
       </c>
       <c r="AM9">
-        <f>LOG(J9)</f>
+        <f t="shared" si="8"/>
         <v>0.95424250943932487</v>
       </c>
       <c r="AP9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="11"/>
         <v>2.1303337684950061</v>
       </c>
       <c r="AQ9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="9"/>
         <v>2.255272505103306</v>
       </c>
       <c r="AR9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="9"/>
         <v>1.4313637641589874</v>
       </c>
       <c r="AU9">
-        <f t="shared" si="3"/>
+        <f t="shared" si="12"/>
         <v>1.7923916894982539</v>
       </c>
       <c r="AV9">
-        <f t="shared" si="1"/>
+        <f t="shared" si="10"/>
         <v>2.0644579892269186</v>
       </c>
       <c r="AW9">
-        <f t="shared" si="1"/>
+        <f t="shared" si="10"/>
         <v>1.5440680443502757</v>
       </c>
     </row>
@@ -16186,63 +17350,63 @@
         <v>39</v>
       </c>
       <c r="AA10">
-        <f>LOG(B10)</f>
+        <f t="shared" si="0"/>
         <v>3.5400790888041729</v>
       </c>
       <c r="AB10">
-        <f>LOG(C10)</f>
+        <f t="shared" si="1"/>
         <v>4.875923205849455</v>
       </c>
       <c r="AC10">
-        <f>LOG(D10)</f>
+        <f t="shared" si="2"/>
         <v>5.0521589186766507</v>
       </c>
       <c r="AF10">
-        <f>LOG(E10)</f>
+        <f t="shared" si="3"/>
         <v>2.1271047983648077</v>
       </c>
       <c r="AG10">
-        <f>LOG(F10)</f>
+        <f t="shared" si="4"/>
         <v>2.4132997640812519</v>
       </c>
       <c r="AH10">
-        <f>LOG(G10)</f>
+        <f t="shared" si="5"/>
         <v>1.8692317197309762</v>
       </c>
       <c r="AK10">
-        <f>LOG(H10)</f>
+        <f t="shared" si="6"/>
         <v>1.8260748027008264</v>
       </c>
       <c r="AL10">
-        <f>LOG(I10)</f>
+        <f t="shared" si="7"/>
         <v>2.1072099696478683</v>
       </c>
       <c r="AM10">
-        <f>LOG(J10)</f>
+        <f t="shared" si="8"/>
         <v>1</v>
       </c>
       <c r="AP10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="11"/>
         <v>2.1760912590556813</v>
       </c>
       <c r="AQ10">
-        <f t="shared" si="0"/>
+        <f t="shared" si="9"/>
         <v>2.3010299956639813</v>
       </c>
       <c r="AR10">
-        <f t="shared" si="0"/>
+        <f t="shared" si="9"/>
         <v>1.4771212547196624</v>
       </c>
       <c r="AU10">
-        <f t="shared" si="3"/>
+        <f t="shared" si="12"/>
         <v>1.8388490907372552</v>
       </c>
       <c r="AV10">
-        <f t="shared" si="1"/>
+        <f t="shared" si="10"/>
         <v>2.1105897102992488</v>
       </c>
       <c r="AW10">
-        <f t="shared" si="1"/>
+        <f t="shared" si="10"/>
         <v>1.5910646070264991</v>
       </c>
     </row>
@@ -16296,63 +17460,63 @@
         <v>43</v>
       </c>
       <c r="AA11">
-        <f>LOG(B11)</f>
+        <f t="shared" si="0"/>
         <v>3.6929350025311378</v>
       </c>
       <c r="AB11">
-        <f>LOG(C11)</f>
+        <f t="shared" si="1"/>
         <v>5.0613695329844326</v>
       </c>
       <c r="AC11">
-        <f>LOG(D11)</f>
+        <f t="shared" si="2"/>
         <v>5.242953663274962</v>
       </c>
       <c r="AF11">
-        <f>LOG(E11)</f>
+        <f t="shared" si="3"/>
         <v>2.1702617153949575</v>
       </c>
       <c r="AG11">
-        <f>LOG(F11)</f>
+        <f t="shared" si="4"/>
         <v>2.4638929889859074</v>
       </c>
       <c r="AH11">
-        <f>LOG(G11)</f>
+        <f t="shared" si="5"/>
         <v>1.9395192526186185</v>
       </c>
       <c r="AK11">
-        <f>LOG(H11)</f>
+        <f t="shared" si="6"/>
         <v>1.8692317197309762</v>
       </c>
       <c r="AL11">
-        <f>LOG(I11)</f>
+        <f t="shared" si="7"/>
         <v>2.1492191126553797</v>
       </c>
       <c r="AM11">
-        <f>LOG(J11)</f>
+        <f t="shared" si="8"/>
         <v>1.0413926851582251</v>
       </c>
       <c r="AP11">
-        <f t="shared" si="2"/>
+        <f t="shared" si="11"/>
         <v>2.2174839442139063</v>
       </c>
       <c r="AQ11">
-        <f t="shared" si="0"/>
+        <f t="shared" si="9"/>
         <v>2.3424226808222062</v>
       </c>
       <c r="AR11">
-        <f t="shared" si="0"/>
+        <f t="shared" si="9"/>
         <v>1.5185139398778875</v>
       </c>
       <c r="AU11">
-        <f t="shared" si="3"/>
+        <f t="shared" si="12"/>
         <v>1.8808135922807914</v>
       </c>
       <c r="AV11">
-        <f t="shared" si="1"/>
+        <f t="shared" si="10"/>
         <v>2.1522883443830563</v>
       </c>
       <c r="AW11">
-        <f t="shared" si="1"/>
+        <f t="shared" si="10"/>
         <v>1.6334684555795864</v>
       </c>
     </row>
@@ -16406,63 +17570,63 @@
         <v>47</v>
       </c>
       <c r="AA12">
-        <f>LOG(B12)</f>
+        <f t="shared" si="0"/>
         <v>3.8334658601706924</v>
       </c>
       <c r="AB12">
-        <f>LOG(C12)</f>
+        <f t="shared" si="1"/>
         <v>5.2319637524310654</v>
       </c>
       <c r="AC12">
-        <f>LOG(D12)</f>
+        <f t="shared" si="2"/>
         <v>5.4183046065321445</v>
       </c>
       <c r="AF12">
-        <f>LOG(E12)</f>
+        <f t="shared" si="3"/>
         <v>2.2095150145426308</v>
       </c>
       <c r="AG12">
-        <f>LOG(F12)</f>
+        <f t="shared" si="4"/>
         <v>2.510545010206612</v>
       </c>
       <c r="AH12">
-        <f>LOG(G12)</f>
+        <f t="shared" si="5"/>
         <v>2.0043213737826426</v>
       </c>
       <c r="AK12">
-        <f>LOG(H12)</f>
+        <f t="shared" si="6"/>
         <v>1.9084850188786497</v>
       </c>
       <c r="AL12">
-        <f>LOG(I12)</f>
+        <f t="shared" si="7"/>
         <v>2.1875207208364631</v>
       </c>
       <c r="AM12">
-        <f>LOG(J12)</f>
+        <f t="shared" si="8"/>
         <v>1.0791812460476249</v>
       </c>
       <c r="AP12">
-        <f t="shared" si="2"/>
+        <f t="shared" si="11"/>
         <v>2.255272505103306</v>
       </c>
       <c r="AQ12">
-        <f t="shared" si="0"/>
+        <f t="shared" si="9"/>
         <v>2.3802112417116059</v>
       </c>
       <c r="AR12">
-        <f t="shared" si="0"/>
+        <f t="shared" si="9"/>
         <v>1.5563025007672873</v>
       </c>
       <c r="AU12">
-        <f t="shared" si="3"/>
+        <f t="shared" si="12"/>
         <v>1.919078092376074</v>
       </c>
       <c r="AV12">
-        <f t="shared" si="1"/>
+        <f t="shared" si="10"/>
         <v>2.1903316981702914</v>
       </c>
       <c r="AW12">
-        <f t="shared" si="1"/>
+        <f t="shared" si="10"/>
         <v>1.6720978579357175</v>
       </c>
     </row>
@@ -16516,63 +17680,63 @@
         <v>51</v>
       </c>
       <c r="AA13">
-        <f>LOG(B13)</f>
+        <f t="shared" si="0"/>
         <v>3.9635044994142907</v>
       </c>
       <c r="AB13">
-        <f>LOG(C13)</f>
+        <f t="shared" si="1"/>
         <v>5.389936494915041</v>
       </c>
       <c r="AC13">
-        <f>LOG(D13)</f>
+        <f t="shared" si="2"/>
         <v>5.5805292569017242</v>
       </c>
       <c r="AF13">
-        <f>LOG(E13)</f>
+        <f t="shared" si="3"/>
         <v>2.2455126678141499</v>
       </c>
       <c r="AG13">
-        <f>LOG(F13)</f>
+        <f t="shared" si="4"/>
         <v>2.5538830266438746</v>
       </c>
       <c r="AH13">
-        <f>LOG(G13)</f>
+        <f t="shared" si="5"/>
         <v>2.0644579892269186</v>
       </c>
       <c r="AK13">
-        <f>LOG(H13)</f>
+        <f t="shared" si="6"/>
         <v>1.9444826721501687</v>
       </c>
       <c r="AL13">
-        <f>LOG(I13)</f>
+        <f t="shared" si="7"/>
         <v>2.2227164711475833</v>
       </c>
       <c r="AM13">
-        <f>LOG(J13)</f>
+        <f t="shared" si="8"/>
         <v>1.1139433523068367</v>
       </c>
       <c r="AP13">
-        <f t="shared" si="2"/>
+        <f t="shared" si="11"/>
         <v>2.2900346113625178</v>
       </c>
       <c r="AQ13">
-        <f t="shared" si="0"/>
+        <f t="shared" si="9"/>
         <v>2.4149733479708178</v>
       </c>
       <c r="AR13">
-        <f t="shared" si="0"/>
+        <f t="shared" si="9"/>
         <v>1.5910646070264991</v>
       </c>
       <c r="AU13">
-        <f t="shared" si="3"/>
+        <f t="shared" si="12"/>
         <v>1.954242509439325</v>
       </c>
       <c r="AV13">
-        <f t="shared" si="1"/>
+        <f t="shared" si="10"/>
         <v>2.2253092817258628</v>
       </c>
       <c r="AW13">
-        <f t="shared" si="1"/>
+        <f t="shared" si="10"/>
         <v>1.7075701760979363</v>
       </c>
     </row>
@@ -16626,63 +17790,63 @@
         <v>55</v>
       </c>
       <c r="AA14">
-        <f>LOG(B14)</f>
+        <f t="shared" si="0"/>
         <v>4.0845047832462278</v>
       </c>
       <c r="AB14">
-        <f>LOG(C14)</f>
+        <f t="shared" si="1"/>
         <v>5.5370467492426405</v>
       </c>
       <c r="AC14">
-        <f>LOG(D14)</f>
+        <f t="shared" si="2"/>
         <v>5.7314590214827037</v>
       </c>
       <c r="AF14">
-        <f>LOG(E14)</f>
+        <f t="shared" si="3"/>
         <v>2.2787536009528289</v>
       </c>
       <c r="AG14">
-        <f>LOG(F14)</f>
+        <f t="shared" si="4"/>
         <v>2.5943925503754266</v>
       </c>
       <c r="AH14">
-        <f>LOG(G14)</f>
+        <f t="shared" si="5"/>
         <v>2.12057393120585</v>
       </c>
       <c r="AK14">
-        <f>LOG(H14)</f>
+        <f t="shared" si="6"/>
         <v>1.9777236052888478</v>
       </c>
       <c r="AL14">
-        <f>LOG(I14)</f>
+        <f t="shared" si="7"/>
         <v>2.255272505103306</v>
       </c>
       <c r="AM14">
-        <f>LOG(J14)</f>
+        <f t="shared" si="8"/>
         <v>1.146128035678238</v>
       </c>
       <c r="AP14">
-        <f t="shared" si="2"/>
+        <f t="shared" si="11"/>
         <v>2.3222192947339191</v>
       </c>
       <c r="AQ14">
-        <f t="shared" si="0"/>
+        <f t="shared" si="9"/>
         <v>2.4471580313422194</v>
       </c>
       <c r="AR14">
-        <f t="shared" si="0"/>
+        <f t="shared" si="9"/>
         <v>1.6232492903979006</v>
       </c>
       <c r="AU14">
-        <f t="shared" si="3"/>
+        <f t="shared" si="12"/>
         <v>1.9867717342662448</v>
       </c>
       <c r="AV14">
-        <f t="shared" si="1"/>
+        <f t="shared" si="10"/>
         <v>2.2576785748691846</v>
       </c>
       <c r="AW14">
-        <f t="shared" si="1"/>
+        <f t="shared" si="10"/>
         <v>1.7403626894942439</v>
       </c>
     </row>
@@ -16736,63 +17900,63 @@
         <v>59</v>
       </c>
       <c r="AA15">
-        <f>LOG(B15)</f>
+        <f t="shared" si="0"/>
         <v>4.1976388755555698</v>
       </c>
       <c r="AB15">
-        <f>LOG(C15)</f>
+        <f t="shared" si="1"/>
         <v>5.6747068607520914</v>
       </c>
       <c r="AC15">
-        <f>LOG(D15)</f>
+        <f t="shared" si="2"/>
         <v>5.8725664726779767</v>
       </c>
       <c r="AF15">
-        <f>LOG(E15)</f>
+        <f t="shared" si="3"/>
         <v>2.3096301674258988</v>
       </c>
       <c r="AG15">
-        <f>LOG(F15)</f>
+        <f t="shared" si="4"/>
         <v>2.6324572921847245</v>
       </c>
       <c r="AH15">
-        <f>LOG(G15)</f>
+        <f t="shared" si="5"/>
         <v>2.173186268412274</v>
       </c>
       <c r="AK15">
-        <f>LOG(H15)</f>
+        <f t="shared" si="6"/>
         <v>2.0086001717619175</v>
       </c>
       <c r="AL15">
-        <f>LOG(I15)</f>
+        <f t="shared" si="7"/>
         <v>2.2855573090077739</v>
       </c>
       <c r="AM15">
-        <f>LOG(J15)</f>
+        <f t="shared" si="8"/>
         <v>1.1760912590556813</v>
       </c>
       <c r="AP15">
-        <f t="shared" si="2"/>
+        <f t="shared" si="11"/>
         <v>2.3521825181113627</v>
       </c>
       <c r="AQ15">
-        <f t="shared" si="0"/>
+        <f t="shared" si="9"/>
         <v>2.4771212547196626</v>
       </c>
       <c r="AR15">
-        <f t="shared" si="0"/>
+        <f t="shared" si="9"/>
         <v>1.6532125137753437</v>
       </c>
       <c r="AU15">
-        <f t="shared" si="3"/>
+        <f t="shared" si="12"/>
         <v>2.0170333392987803</v>
       </c>
       <c r="AV15">
-        <f t="shared" si="1"/>
+        <f t="shared" si="10"/>
         <v>2.287801729930226</v>
       </c>
       <c r="AW15">
-        <f t="shared" si="1"/>
+        <f t="shared" si="10"/>
         <v>1.7708520116421442</v>
       </c>
     </row>
@@ -16846,63 +18010,63 @@
         <v>63</v>
       </c>
       <c r="AA16">
-        <f>LOG(B16)</f>
+        <f t="shared" si="0"/>
         <v>4.3038653488427041</v>
       </c>
       <c r="AB16">
-        <f>LOG(C16)</f>
+        <f t="shared" si="1"/>
         <v>5.8040685213250036</v>
       </c>
       <c r="AC16">
-        <f>LOG(D16)</f>
+        <f t="shared" si="2"/>
         <v>6.0050534670785991</v>
       </c>
       <c r="AF16">
-        <f>LOG(E16)</f>
+        <f t="shared" si="3"/>
         <v>2.3384564936046046</v>
       </c>
       <c r="AG16">
-        <f>LOG(F16)</f>
+        <f t="shared" si="4"/>
         <v>2.6683859166900001</v>
       </c>
       <c r="AH16">
-        <f>LOG(G16)</f>
+        <f t="shared" si="5"/>
         <v>2.2227164711475833</v>
       </c>
       <c r="AK16">
-        <f>LOG(H16)</f>
+        <f t="shared" si="6"/>
         <v>2.0374264979406238</v>
       </c>
       <c r="AL16">
-        <f>LOG(I16)</f>
+        <f t="shared" si="7"/>
         <v>2.3138672203691533</v>
       </c>
       <c r="AM16">
-        <f>LOG(J16)</f>
+        <f t="shared" si="8"/>
         <v>1.2041199826559248</v>
       </c>
       <c r="AP16">
-        <f t="shared" si="2"/>
+        <f t="shared" si="11"/>
         <v>2.3802112417116059</v>
       </c>
       <c r="AQ16">
-        <f t="shared" si="0"/>
+        <f t="shared" si="9"/>
         <v>2.5051499783199058</v>
       </c>
       <c r="AR16">
-        <f t="shared" si="0"/>
+        <f t="shared" si="9"/>
         <v>1.6812412373755872</v>
       </c>
       <c r="AU16">
-        <f t="shared" si="3"/>
+        <f t="shared" si="12"/>
         <v>2.0453229787866576</v>
       </c>
       <c r="AV16">
-        <f t="shared" si="1"/>
+        <f t="shared" si="10"/>
         <v>2.3159703454569178</v>
       </c>
       <c r="AW16">
-        <f t="shared" si="1"/>
+        <f t="shared" si="10"/>
         <v>1.7993405494535817</v>
       </c>
     </row>
@@ -16956,63 +18120,63 @@
         <v>67</v>
       </c>
       <c r="AA17">
-        <f>LOG(B17)</f>
+        <f t="shared" si="0"/>
         <v>4.4039779636693543</v>
       </c>
       <c r="AB17">
-        <f>LOG(C17)</f>
+        <f t="shared" si="1"/>
         <v>5.926083542306575</v>
       </c>
       <c r="AC17">
-        <f>LOG(D17)</f>
+        <f t="shared" si="2"/>
         <v>6.1299137474529397</v>
       </c>
       <c r="AF17">
-        <f>LOG(E17)</f>
+        <f t="shared" si="3"/>
         <v>2.3654879848908998</v>
       </c>
       <c r="AG17">
-        <f>LOG(F17)</f>
+        <f t="shared" si="4"/>
         <v>2.7024305364455254</v>
       </c>
       <c r="AH17">
-        <f>LOG(G17)</f>
+        <f t="shared" si="5"/>
         <v>2.2695129442179165</v>
       </c>
       <c r="AK17">
-        <f>LOG(H17)</f>
+        <f t="shared" si="6"/>
         <v>2.0644579892269186</v>
       </c>
       <c r="AL17">
-        <f>LOG(I17)</f>
+        <f t="shared" si="7"/>
         <v>2.3404441148401185</v>
       </c>
       <c r="AM17">
-        <f>LOG(J17)</f>
+        <f t="shared" si="8"/>
         <v>1.2304489213782739</v>
       </c>
       <c r="AP17">
-        <f t="shared" si="2"/>
+        <f t="shared" si="11"/>
         <v>2.406540180433955</v>
       </c>
       <c r="AQ17">
-        <f t="shared" si="0"/>
+        <f t="shared" si="9"/>
         <v>2.5314789170422549</v>
       </c>
       <c r="AR17">
-        <f t="shared" si="0"/>
+        <f t="shared" si="9"/>
         <v>1.7075701760979363</v>
       </c>
       <c r="AU17">
-        <f t="shared" si="3"/>
+        <f t="shared" si="12"/>
         <v>2.0718820073061255</v>
       </c>
       <c r="AV17">
-        <f t="shared" si="1"/>
+        <f t="shared" si="10"/>
         <v>2.3424226808222062</v>
       </c>
       <c r="AW17">
-        <f t="shared" si="1"/>
+        <f t="shared" si="10"/>
         <v>1.8260748027008264</v>
       </c>
     </row>
@@ -17066,63 +18230,63 @@
         <v>71</v>
       </c>
       <c r="AA18">
-        <f>LOG(B18)</f>
+        <f t="shared" si="0"/>
         <v>4.4986413188336947</v>
       </c>
       <c r="AB18">
-        <f>LOG(C18)</f>
+        <f t="shared" si="1"/>
         <v>6.0415478190213152</v>
       </c>
       <c r="AC18">
-        <f>LOG(D18)</f>
+        <f t="shared" si="2"/>
         <v>6.2479784189776355</v>
       </c>
       <c r="AF18">
-        <f>LOG(E18)</f>
+        <f t="shared" si="3"/>
         <v>2.3909351071033793</v>
       </c>
       <c r="AG18">
-        <f>LOG(F18)</f>
+        <f t="shared" si="4"/>
         <v>2.7347998295888472</v>
       </c>
       <c r="AH18">
-        <f>LOG(G18)</f>
+        <f t="shared" si="5"/>
         <v>2.3138672203691533</v>
       </c>
       <c r="AK18">
-        <f>LOG(H18)</f>
+        <f t="shared" si="6"/>
         <v>2.0899051114393981</v>
       </c>
       <c r="AL18">
-        <f>LOG(I18)</f>
+        <f t="shared" si="7"/>
         <v>2.3654879848908998</v>
       </c>
       <c r="AM18">
-        <f>LOG(J18)</f>
+        <f t="shared" si="8"/>
         <v>1.255272505103306</v>
       </c>
       <c r="AP18">
-        <f t="shared" si="2"/>
+        <f t="shared" si="11"/>
         <v>2.4313637641589874</v>
       </c>
       <c r="AQ18">
-        <f t="shared" ref="AQ18:AQ20" si="4">LOG(L18)</f>
+        <f t="shared" ref="AQ18:AQ20" si="13">LOG(L18)</f>
         <v>2.5563025007672873</v>
       </c>
       <c r="AR18">
-        <f t="shared" ref="AR18:AR20" si="5">LOG(M18)</f>
+        <f t="shared" ref="AR18:AR20" si="14">LOG(M18)</f>
         <v>1.7323937598229686</v>
       </c>
       <c r="AU18">
-        <f t="shared" si="3"/>
+        <f t="shared" si="12"/>
         <v>2.0969100130080562</v>
       </c>
       <c r="AV18">
-        <f t="shared" ref="AV18:AV20" si="6">LOG(O18)</f>
+        <f t="shared" ref="AV18:AV20" si="15">LOG(O18)</f>
         <v>2.3673559210260189</v>
       </c>
       <c r="AW18">
-        <f t="shared" ref="AW18:AW20" si="7">LOG(P18)</f>
+        <f t="shared" ref="AW18:AW20" si="16">LOG(P18)</f>
         <v>1.8512583487190752</v>
       </c>
     </row>
@@ -17176,63 +18340,63 @@
         <v>75</v>
       </c>
       <c r="AA19">
-        <f>LOG(B19)</f>
+        <f t="shared" si="0"/>
         <v>4.5884173812019249</v>
       </c>
       <c r="AB19">
-        <f>LOG(C19)</f>
+        <f t="shared" si="1"/>
         <v>6.151133789808104</v>
       </c>
       <c r="AC19">
-        <f>LOG(D19)</f>
+        <f t="shared" si="2"/>
         <v>6.3599496355798379</v>
       </c>
       <c r="AF19">
-        <f>LOG(E19)</f>
+        <f t="shared" si="3"/>
         <v>2.4149733479708178</v>
       </c>
       <c r="AG19">
-        <f>LOG(F19)</f>
+        <f t="shared" si="4"/>
         <v>2.7656685547590141</v>
       </c>
       <c r="AH19">
-        <f>LOG(G19)</f>
+        <f t="shared" si="5"/>
         <v>2.3560258571931225</v>
       </c>
       <c r="AK19">
-        <f>LOG(H19)</f>
+        <f t="shared" si="6"/>
         <v>2.1139433523068369</v>
       </c>
       <c r="AL19">
-        <f>LOG(I19)</f>
+        <f t="shared" si="7"/>
         <v>2.3891660843645326</v>
       </c>
       <c r="AM19">
-        <f>LOG(J19)</f>
+        <f t="shared" si="8"/>
         <v>1.2787536009528289</v>
       </c>
       <c r="AP19">
-        <f t="shared" si="2"/>
+        <f t="shared" si="11"/>
         <v>2.4548448600085102</v>
       </c>
       <c r="AQ19">
-        <f t="shared" si="4"/>
+        <f t="shared" si="13"/>
         <v>2.5797835966168101</v>
       </c>
       <c r="AR19">
-        <f t="shared" si="5"/>
+        <f t="shared" si="14"/>
         <v>1.7558748556724915</v>
       </c>
       <c r="AU19">
-        <f t="shared" si="3"/>
+        <f t="shared" si="12"/>
         <v>2.12057393120585</v>
       </c>
       <c r="AV19">
-        <f t="shared" si="6"/>
+        <f t="shared" si="15"/>
         <v>2.3909351071033793</v>
       </c>
       <c r="AW19">
-        <f t="shared" si="7"/>
+        <f t="shared" si="16"/>
         <v>1.8750612633917001</v>
       </c>
     </row>
@@ -17286,63 +18450,63 @@
         <v>79</v>
       </c>
       <c r="AA20">
-        <f>LOG(B20)</f>
+        <f t="shared" si="0"/>
         <v>4.6737855508358148</v>
       </c>
       <c r="AB20">
-        <f>LOG(C20)</f>
+        <f t="shared" si="1"/>
         <v>6.2554148338586577</v>
       </c>
       <c r="AC20">
-        <f>LOG(D20)</f>
+        <f t="shared" si="2"/>
         <v>6.4664259866779652</v>
       </c>
       <c r="AF20">
-        <f>LOG(E20)</f>
+        <f t="shared" si="3"/>
         <v>2.4377505628203879</v>
       </c>
       <c r="AG20">
-        <f>LOG(F20)</f>
+        <f t="shared" si="4"/>
         <v>2.7951845896824241</v>
       </c>
       <c r="AH20">
-        <f>LOG(G20)</f>
+        <f t="shared" si="5"/>
         <v>2.3961993470957363</v>
       </c>
       <c r="AK20">
-        <f>LOG(H20)</f>
+        <f t="shared" si="6"/>
         <v>2.1367205671564067</v>
       </c>
       <c r="AL20">
-        <f>LOG(I20)</f>
+        <f t="shared" si="7"/>
         <v>2.4116197059632301</v>
       </c>
       <c r="AM20">
-        <f>LOG(J20)</f>
+        <f t="shared" si="8"/>
         <v>1.3010299956639813</v>
       </c>
       <c r="AP20">
-        <f t="shared" si="2"/>
+        <f t="shared" si="11"/>
         <v>2.4771212547196626</v>
       </c>
       <c r="AQ20">
-        <f t="shared" si="4"/>
+        <f t="shared" si="13"/>
         <v>2.6020599913279625</v>
       </c>
       <c r="AR20">
-        <f t="shared" si="5"/>
+        <f t="shared" si="14"/>
         <v>1.7781512503836436</v>
       </c>
       <c r="AU20">
-        <f t="shared" si="3"/>
+        <f t="shared" si="12"/>
         <v>2.143014800254095</v>
       </c>
       <c r="AV20">
-        <f t="shared" si="6"/>
+        <f t="shared" si="15"/>
         <v>2.4132997640812519</v>
       </c>
       <c r="AW20">
-        <f t="shared" si="7"/>
+        <f t="shared" si="16"/>
         <v>1.8976270912904414</v>
       </c>
     </row>

</xml_diff>